<commit_message>
Rev B: verify JLC SMT J1/L1, tighten buck routing and audit 3A/GND (NO-GO)
</commit_message>
<xml_diff>
--- a/manufacturing/Rev_B/REVIEW_ONLY_NOT_FOR_FAB/FT2D_RevB_SMT_sourcing_DRAFT.xlsx
+++ b/manufacturing/Rev_B/REVIEW_ONLY_NOT_FOR_FAB/FT2D_RevB_SMT_sourcing_DRAFT.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="R220afe0aa4074597"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM review" sheetId="2" r:id="R4fc80745e7c340c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPL preview" sheetId="3" r:id="Re154214f680d4cc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="R78b72b3de5e84521"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM review" sheetId="2" r:id="R77e2722ba1ff463f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPL preview" sheetId="3" r:id="R72f6cb30431a4032"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="0.000"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -75,8 +75,13 @@
       <x:color rgb="FFB91C1C"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF065F46"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -98,6 +103,11 @@
         <x:fgColor rgb="FFFEF3C7"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD1FAE5"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -111,7 +121,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="19">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -127,6 +137,8 @@
     <x:xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
@@ -366,7 +378,7 @@
         <x:v>PCB DRC</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>1 library mismatch; 4 unconnected GND regions</x:v>
+        <x:v>0 violations; 5 unconnected GND items (NO-GO)</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -374,7 +386,7 @@
         <x:v>3A power copper</x:v>
       </x:c>
       <x:c r="B9" s="6" t="str">
-        <x:v>Long runs still 0.6mm; repour/reroute required</x:v>
+        <x:v>Top copper corridors target 1.6-2.0mm; necks and thermal return NOT signed off</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -387,10 +399,10 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="7" t="str">
-        <x:v>USB-C connector</x:v>
+        <x:v>J1 / L1</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
-        <x:v>Listed as through-hole / wave solder, not SMT</x:v>
+        <x:v>HRO C165948 and JIERR C53463013 selected; OEM pad dimensions checked</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -398,7 +410,7 @@
         <x:v>Placement file</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
-        <x:v>Preview only; visually verify Y sign/rotation in JLC</x:v>
+        <x:v>53 SMT positions; -90deg USB-C placement &amp; Y sign need JLC review</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -629,10 +641,10 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="9" t="str">
-        <x:v>C12</x:v>
+        <x:v>C11</x:v>
       </x:c>
       <x:c r="B8" s="9" t="str">
-        <x:v>100n_50V</x:v>
+        <x:v>10p_DNP</x:v>
       </x:c>
       <x:c r="C8" s="9" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
@@ -643,21 +655,21 @@
       <x:c r="E8" s="9" t="str"/>
       <x:c r="F8" s="9" t="str"/>
       <x:c r="G8" s="9" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="H8" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>Do not place</x:v>
+      </x:c>
+      <x:c r="H8" s="9" t="str">
+        <x:v>DNP</x:v>
       </x:c>
       <x:c r="I8" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Deliberately omitted from SMT CPL</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>YES</x:v>
+        <x:v>NO</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="9" t="str">
-        <x:v>C13</x:v>
+        <x:v>C12</x:v>
       </x:c>
       <x:c r="B9" s="9" t="str">
         <x:v>100n_50V</x:v>
@@ -685,13 +697,13 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="9" t="str">
-        <x:v>C14</x:v>
+        <x:v>C13</x:v>
       </x:c>
       <x:c r="B10" s="9" t="str">
-        <x:v>10u_50V</x:v>
+        <x:v>100n_50V</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>Capacitor_SMD:C_1210_3225Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D10" s="10" t="n">
         <x:v>1</x:v>
@@ -713,7 +725,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="9" t="str">
-        <x:v>C15</x:v>
+        <x:v>C14</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
         <x:v>10u_50V</x:v>
@@ -741,7 +753,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="9" t="str">
-        <x:v>C16</x:v>
+        <x:v>C15</x:v>
       </x:c>
       <x:c r="B12" s="9" t="str">
         <x:v>10u_50V</x:v>
@@ -769,7 +781,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="9" t="str">
-        <x:v>C17</x:v>
+        <x:v>C16</x:v>
       </x:c>
       <x:c r="B13" s="9" t="str">
         <x:v>10u_50V</x:v>
@@ -797,29 +809,27 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="9" t="str">
-        <x:v>C18</x:v>
+        <x:v>C17</x:v>
       </x:c>
       <x:c r="B14" s="9" t="str">
-        <x:v>EEHZL1V470R_47u</x:v>
+        <x:v>10u_50V</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>Capacitor_SMD:CP_Elec_5x5.8</x:v>
+        <x:v>Capacitor_SMD:C_1210_3225Metric</x:v>
       </x:c>
       <x:c r="D14" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E14" s="9" t="str">
-        <x:v>EEHZL1V470R</x:v>
-      </x:c>
+      <x:c r="E14" s="9" t="str"/>
       <x:c r="F14" s="9" t="str"/>
       <x:c r="G14" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="H14" s="14" t="str">
-        <x:v>NO CONFIRMED SKU</x:v>
+      <x:c r="H14" s="12" t="str">
+        <x:v>SKU NOT ASSIGNED</x:v>
       </x:c>
       <x:c r="I14" s="9" t="str">
-        <x:v>Check ESR, voltage and physical fit</x:v>
+        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
       </x:c>
       <x:c r="J14" s="9" t="str">
         <x:v>YES</x:v>
@@ -827,27 +837,29 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="9" t="str">
-        <x:v>C19</x:v>
+        <x:v>C18</x:v>
       </x:c>
       <x:c r="B15" s="9" t="str">
-        <x:v>100n_16V</x:v>
+        <x:v>EEHZL1V470R_47u</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
+        <x:v>Capacitor_SMD:CP_Elec_5x5.8</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E15" s="9" t="str"/>
+      <x:c r="E15" s="9" t="str">
+        <x:v>EEHZL1V470R</x:v>
+      </x:c>
       <x:c r="F15" s="9" t="str"/>
       <x:c r="G15" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="H15" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+      <x:c r="H15" s="14" t="str">
+        <x:v>NO CONFIRMED SKU</x:v>
       </x:c>
       <x:c r="I15" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Check ESR, voltage and physical fit</x:v>
       </x:c>
       <x:c r="J15" s="9" t="str">
         <x:v>YES</x:v>
@@ -855,13 +867,13 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="9" t="str">
-        <x:v>C20</x:v>
+        <x:v>C19</x:v>
       </x:c>
       <x:c r="B16" s="9" t="str">
-        <x:v>47u_25V</x:v>
+        <x:v>100n_16V</x:v>
       </x:c>
       <x:c r="C16" s="9" t="str">
-        <x:v>Capacitor_SMD:C_1210_3225Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D16" s="10" t="n">
         <x:v>1</x:v>
@@ -883,7 +895,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="9" t="str">
-        <x:v>C21</x:v>
+        <x:v>C20</x:v>
       </x:c>
       <x:c r="B17" s="9" t="str">
         <x:v>47u_25V</x:v>
@@ -911,7 +923,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="9" t="str">
-        <x:v>C22</x:v>
+        <x:v>C21</x:v>
       </x:c>
       <x:c r="B18" s="9" t="str">
         <x:v>47u_25V</x:v>
@@ -939,29 +951,27 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="9" t="str">
-        <x:v>C23</x:v>
+        <x:v>C22</x:v>
       </x:c>
       <x:c r="B19" s="9" t="str">
-        <x:v>250AVHT221M0608_220u</x:v>
+        <x:v>47u_25V</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>Capacitor_SMD:CP_Elec_6.3x7.7</x:v>
+        <x:v>Capacitor_SMD:C_1210_3225Metric</x:v>
       </x:c>
       <x:c r="D19" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E19" s="9" t="str">
-        <x:v>250AVHT221M0608</x:v>
-      </x:c>
+      <x:c r="E19" s="9" t="str"/>
       <x:c r="F19" s="9" t="str"/>
       <x:c r="G19" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="H19" s="14" t="str">
-        <x:v>NO CONFIRMED SKU</x:v>
+      <x:c r="H19" s="12" t="str">
+        <x:v>SKU NOT ASSIGNED</x:v>
       </x:c>
       <x:c r="I19" s="9" t="str">
-        <x:v>Verify ESR, ripple current and loop stability</x:v>
+        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
       </x:c>
       <x:c r="J19" s="9" t="str">
         <x:v>YES</x:v>
@@ -969,27 +979,29 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="9" t="str">
-        <x:v>C24</x:v>
+        <x:v>C23</x:v>
       </x:c>
       <x:c r="B20" s="9" t="str">
-        <x:v>100n_25V</x:v>
+        <x:v>250AVHT221M0608_220u</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
+        <x:v>Capacitor_SMD:CP_Elec_6.3x7.7</x:v>
       </x:c>
       <x:c r="D20" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E20" s="9" t="str"/>
+      <x:c r="E20" s="9" t="str">
+        <x:v>250AVHT221M0608</x:v>
+      </x:c>
       <x:c r="F20" s="9" t="str"/>
       <x:c r="G20" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="H20" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+      <x:c r="H20" s="14" t="str">
+        <x:v>NO CONFIRMED SKU</x:v>
       </x:c>
       <x:c r="I20" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Verify ESR, ripple current and loop stability</x:v>
       </x:c>
       <x:c r="J20" s="9" t="str">
         <x:v>YES</x:v>
@@ -997,13 +1009,13 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="9" t="str">
-        <x:v>C25</x:v>
+        <x:v>C24</x:v>
       </x:c>
       <x:c r="B21" s="9" t="str">
-        <x:v>47u_25V</x:v>
+        <x:v>100n_25V</x:v>
       </x:c>
       <x:c r="C21" s="9" t="str">
-        <x:v>Capacitor_SMD:C_1210_3225Metric</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D21" s="10" t="n">
         <x:v>1</x:v>
@@ -1025,13 +1037,13 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="9" t="str">
-        <x:v>C26</x:v>
+        <x:v>C25</x:v>
       </x:c>
       <x:c r="B22" s="9" t="str">
-        <x:v>100n_25V</x:v>
+        <x:v>47u_25V</x:v>
       </x:c>
       <x:c r="C22" s="9" t="str">
-        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
+        <x:v>Capacitor_SMD:C_1210_3225Metric</x:v>
       </x:c>
       <x:c r="D22" s="10" t="n">
         <x:v>1</x:v>
@@ -1053,10 +1065,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="9" t="str">
-        <x:v>C27</x:v>
+        <x:v>C26</x:v>
       </x:c>
       <x:c r="B23" s="9" t="str">
-        <x:v>3n3_25V</x:v>
+        <x:v>100n_25V</x:v>
       </x:c>
       <x:c r="C23" s="9" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
@@ -1081,10 +1093,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="9" t="str">
-        <x:v>C28</x:v>
+        <x:v>C27</x:v>
       </x:c>
       <x:c r="B24" s="9" t="str">
-        <x:v>2n2_10V</x:v>
+        <x:v>3n3_25V</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
         <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
@@ -1109,13 +1121,13 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="9" t="str">
-        <x:v>D1</x:v>
+        <x:v>C28</x:v>
       </x:c>
       <x:c r="B25" s="9" t="str">
-        <x:v>ESDA25P35-1U1M</x:v>
+        <x:v>2n2_10V</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>FT2D:ST_ESDA25P35_1U1M</x:v>
+        <x:v>Capacitor_SMD:C_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D25" s="10" t="n">
         <x:v>1</x:v>
@@ -1132,18 +1144,18 @@
         <x:v>Verify rating, tolerance, land pattern and stock</x:v>
       </x:c>
       <x:c r="J25" s="9" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="9" t="str">
-        <x:v>D2</x:v>
+        <x:v>D1</x:v>
       </x:c>
       <x:c r="B26" s="9" t="str">
-        <x:v>ESDA25W</x:v>
+        <x:v>ESDA25P35-1U1M</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>Package_TO_SOT_SMD:SOT-323_SC-70</x:v>
+        <x:v>FT2D:ST_ESDA25P35_1U1M</x:v>
       </x:c>
       <x:c r="D26" s="10" t="n">
         <x:v>1</x:v>
@@ -1165,29 +1177,27 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="9" t="str">
-        <x:v>F1</x:v>
+        <x:v>D2</x:v>
       </x:c>
       <x:c r="B27" s="9" t="str">
-        <x:v>1206SFS300F/32</x:v>
+        <x:v>ESDA25W</x:v>
       </x:c>
       <x:c r="C27" s="9" t="str">
-        <x:v>Fuse:Fuse_1206_3216Metric</x:v>
+        <x:v>Package_TO_SOT_SMD:SOT-323_SC-70</x:v>
       </x:c>
       <x:c r="D27" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E27" s="9" t="str">
-        <x:v>1206SFS300F/32</x:v>
-      </x:c>
+      <x:c r="E27" s="9" t="str"/>
       <x:c r="F27" s="9" t="str"/>
       <x:c r="G27" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="H27" s="14" t="str">
-        <x:v>NO CONFIRMED SKU</x:v>
+      <x:c r="H27" s="12" t="str">
+        <x:v>SKU NOT ASSIGNED</x:v>
       </x:c>
       <x:c r="I27" s="9" t="str">
-        <x:v>Match voltage/current, I-squared-t and derating</x:v>
+        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
       </x:c>
       <x:c r="J27" s="9" t="str">
         <x:v>YES</x:v>
@@ -1195,91 +1205,91 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="9" t="str">
-        <x:v>J1</x:v>
+        <x:v>F1</x:v>
       </x:c>
       <x:c r="B28" s="9" t="str">
-        <x:v>USB4085-GF-A</x:v>
+        <x:v>1206SFS300F/32</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
-        <x:v>Connector_USB:USB_C_Receptacle_GCT_USB4085</x:v>
+        <x:v>Fuse:Fuse_1206_3216Metric</x:v>
       </x:c>
       <x:c r="D28" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
-        <x:v>USB4085-GF-A</x:v>
-      </x:c>
-      <x:c r="F28" s="9" t="str">
-        <x:v>C7095263</x:v>
-      </x:c>
+        <x:v>1206SFS300F/32</x:v>
+      </x:c>
+      <x:c r="F28" s="9" t="str"/>
       <x:c r="G28" s="9" t="str">
-        <x:v>THT / wave solder</x:v>
+        <x:v>SMT</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>ASSEMBLY MISMATCH</x:v>
+        <x:v>NO CONFIRMED SKU</x:v>
       </x:c>
       <x:c r="I28" s="9" t="str">
-        <x:v>Ask JLC for mixed assembly or change connector</x:v>
+        <x:v>Match voltage/current, I-squared-t and derating</x:v>
       </x:c>
       <x:c r="J28" s="9" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="9" t="str">
-        <x:v>J2</x:v>
+        <x:v>J1</x:v>
       </x:c>
       <x:c r="B29" s="9" t="str">
-        <x:v>PD_PROGRAM_TEST</x:v>
+        <x:v>TYPE-C-31-M-12</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>FT2D:PD_Programming_Pads_1x06_P2p54</x:v>
+        <x:v>Connector_USB:USB_C_Receptacle_HRO_TYPE-C-31-M-12</x:v>
       </x:c>
       <x:c r="D29" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
-        <x:v>Program pads</x:v>
-      </x:c>
-      <x:c r="F29" s="9" t="str"/>
+        <x:v>TYPE-C-31-M-12</x:v>
+      </x:c>
+      <x:c r="F29" s="9" t="str">
+        <x:v>C165948</x:v>
+      </x:c>
       <x:c r="G29" s="9" t="str">
-        <x:v>PCB feature</x:v>
-      </x:c>
-      <x:c r="H29" s="9" t="str">
-        <x:v>NO SMT</x:v>
+        <x:v>SMT with PTH shield stakes</x:v>
+      </x:c>
+      <x:c r="H29" s="16" t="str">
+        <x:v>MODEL / LAND PATTERN VERIFIED</x:v>
       </x:c>
       <x:c r="I29" s="9" t="str">
-        <x:v>2.7V I2C programming pads; omit from SMT order</x:v>
+        <x:v>JLC listed SMT; check -90deg placement and board-edge connector mechanics in assembly preview</x:v>
       </x:c>
       <x:c r="J29" s="9" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="9" t="str">
-        <x:v>J3</x:v>
+        <x:v>J2</x:v>
       </x:c>
       <x:c r="B30" s="9" t="str">
-        <x:v>E-DC-6_PIGTAIL</x:v>
+        <x:v>PD_PROGRAM_TEST</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>FT2D:Wire_Pads_2x_P3mm</x:v>
+        <x:v>FT2D:PD_Programming_Pads_1x06_P2p54</x:v>
       </x:c>
       <x:c r="D30" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E30" s="9" t="str">
-        <x:v>E-DC-6 pigtail</x:v>
+        <x:v>Program pads</x:v>
       </x:c>
       <x:c r="F30" s="9" t="str"/>
       <x:c r="G30" s="9" t="str">
-        <x:v>Manual wire</x:v>
+        <x:v>PCB feature</x:v>
       </x:c>
       <x:c r="H30" s="9" t="str">
         <x:v>NO SMT</x:v>
       </x:c>
       <x:c r="I30" s="9" t="str">
-        <x:v>Verify output polarity and strain relief</x:v>
+        <x:v>2.7V I2C programming pads; omit from SMT order</x:v>
       </x:c>
       <x:c r="J30" s="9" t="str">
         <x:v>NO</x:v>
@@ -1287,31 +1297,29 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="9" t="str">
-        <x:v>L1</x:v>
+        <x:v>J3</x:v>
       </x:c>
       <x:c r="B31" s="9" t="str">
-        <x:v>SRP1238A-100M_10uH</x:v>
+        <x:v>E-DC-6_PIGTAIL</x:v>
       </x:c>
       <x:c r="C31" s="9" t="str">
-        <x:v>FT2D:Bourns_SRP1238A</x:v>
+        <x:v>FT2D:Wire_Pads_2x_P3mm</x:v>
       </x:c>
       <x:c r="D31" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E31" s="9" t="str">
-        <x:v>SRP1238A-100M</x:v>
-      </x:c>
-      <x:c r="F31" s="9" t="str">
-        <x:v>C2041734</x:v>
-      </x:c>
+        <x:v>E-DC-6 pigtail</x:v>
+      </x:c>
+      <x:c r="F31" s="9" t="str"/>
       <x:c r="G31" s="9" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="H31" s="14" t="str">
-        <x:v>OUT OF STOCK RISK</x:v>
+        <x:v>Manual wire</x:v>
+      </x:c>
+      <x:c r="H31" s="9" t="str">
+        <x:v>NO SMT</x:v>
       </x:c>
       <x:c r="I31" s="9" t="str">
-        <x:v>Validate Isat, Irms, DCR and size before substitution</x:v>
+        <x:v>Verify output polarity and strain relief</x:v>
       </x:c>
       <x:c r="J31" s="9" t="str">
         <x:v>NO</x:v>
@@ -1319,59 +1327,63 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="9" t="str">
-        <x:v>Q1</x:v>
+        <x:v>L1</x:v>
       </x:c>
       <x:c r="B32" s="9" t="str">
-        <x:v>STL6P3LLH6</x:v>
+        <x:v>SRG1260-100-M_10uH</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>FT2D:ST_PowerFLAT_3p3_TypeF</x:v>
+        <x:v>FT2D:JIERR_SRG1260_100M</x:v>
       </x:c>
       <x:c r="D32" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
-        <x:v>STL6P3LLH6</x:v>
+        <x:v>SRG1260-100-M</x:v>
       </x:c>
       <x:c r="F32" s="9" t="str">
-        <x:v>C457492</x:v>
+        <x:v>C53463013</x:v>
       </x:c>
       <x:c r="G32" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
-      <x:c r="H32" s="12" t="str">
-        <x:v>SKU CANDIDATE</x:v>
+      <x:c r="H32" s="16" t="str">
+        <x:v>MODEL / LAND PATTERN VERIFIED</x:v>
       </x:c>
       <x:c r="I32" s="9" t="str">
-        <x:v>Verify PowerFLAT footprint</x:v>
+        <x:v>10uH; Isat 14A typ; Idc 11A typ; DCR 25mOhm max; 6.0mm max height</x:v>
       </x:c>
       <x:c r="J32" s="9" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="9" t="str">
-        <x:v>R1</x:v>
+        <x:v>Q1</x:v>
       </x:c>
       <x:c r="B33" s="9" t="str">
-        <x:v>10k</x:v>
+        <x:v>STL6P3LLH6</x:v>
       </x:c>
       <x:c r="C33" s="9" t="str">
-        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
+        <x:v>FT2D:ST_PowerFLAT_3p3_TypeF</x:v>
       </x:c>
       <x:c r="D33" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E33" s="9" t="str"/>
-      <x:c r="F33" s="9" t="str"/>
+      <x:c r="E33" s="9" t="str">
+        <x:v>STL6P3LLH6</x:v>
+      </x:c>
+      <x:c r="F33" s="9" t="str">
+        <x:v>C457492</x:v>
+      </x:c>
       <x:c r="G33" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H33" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>SKU CANDIDATE</x:v>
       </x:c>
       <x:c r="I33" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Verify PowerFLAT footprint</x:v>
       </x:c>
       <x:c r="J33" s="9" t="str">
         <x:v>YES</x:v>
@@ -1379,10 +1391,10 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="9" t="str">
-        <x:v>R2</x:v>
+        <x:v>R1</x:v>
       </x:c>
       <x:c r="B34" s="9" t="str">
-        <x:v>4k7</x:v>
+        <x:v>10k</x:v>
       </x:c>
       <x:c r="C34" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1407,7 +1419,7 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="9" t="str">
-        <x:v>R3</x:v>
+        <x:v>R2</x:v>
       </x:c>
       <x:c r="B35" s="9" t="str">
         <x:v>4k7</x:v>
@@ -1435,10 +1447,10 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="9" t="str">
-        <x:v>R4</x:v>
+        <x:v>R3</x:v>
       </x:c>
       <x:c r="B36" s="9" t="str">
-        <x:v>1k</x:v>
+        <x:v>4k7</x:v>
       </x:c>
       <x:c r="C36" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1463,10 +1475,10 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="9" t="str">
-        <x:v>R5</x:v>
+        <x:v>R4</x:v>
       </x:c>
       <x:c r="B37" s="9" t="str">
-        <x:v>22k</x:v>
+        <x:v>1k</x:v>
       </x:c>
       <x:c r="C37" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1491,10 +1503,10 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="9" t="str">
-        <x:v>R6</x:v>
+        <x:v>R5</x:v>
       </x:c>
       <x:c r="B38" s="9" t="str">
-        <x:v>470R</x:v>
+        <x:v>22k</x:v>
       </x:c>
       <x:c r="C38" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1519,10 +1531,10 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="9" t="str">
-        <x:v>R7</x:v>
+        <x:v>R6</x:v>
       </x:c>
       <x:c r="B39" s="9" t="str">
-        <x:v>100k</x:v>
+        <x:v>470R</x:v>
       </x:c>
       <x:c r="C39" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1547,10 +1559,10 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="9" t="str">
-        <x:v>R12</x:v>
+        <x:v>R7</x:v>
       </x:c>
       <x:c r="B40" s="9" t="str">
-        <x:v>100k_0.1%</x:v>
+        <x:v>100k</x:v>
       </x:c>
       <x:c r="C40" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1575,10 +1587,10 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="9" t="str">
-        <x:v>R13</x:v>
+        <x:v>R12</x:v>
       </x:c>
       <x:c r="B41" s="9" t="str">
-        <x:v>8k66_0.1%</x:v>
+        <x:v>100k_0.1%</x:v>
       </x:c>
       <x:c r="C41" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1603,10 +1615,10 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="9" t="str">
-        <x:v>R15</x:v>
+        <x:v>R13</x:v>
       </x:c>
       <x:c r="B42" s="9" t="str">
-        <x:v>100k</x:v>
+        <x:v>8k66_0.1%</x:v>
       </x:c>
       <x:c r="C42" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1631,10 +1643,10 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="9" t="str">
-        <x:v>R16</x:v>
+        <x:v>R14</x:v>
       </x:c>
       <x:c r="B43" s="9" t="str">
-        <x:v>33k2</x:v>
+        <x:v>1k_DNP</x:v>
       </x:c>
       <x:c r="C43" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1645,24 +1657,24 @@
       <x:c r="E43" s="9" t="str"/>
       <x:c r="F43" s="9" t="str"/>
       <x:c r="G43" s="9" t="str">
-        <x:v>SMT</x:v>
-      </x:c>
-      <x:c r="H43" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>Do not place</x:v>
+      </x:c>
+      <x:c r="H43" s="9" t="str">
+        <x:v>DNP</x:v>
       </x:c>
       <x:c r="I43" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Deliberately omitted from SMT CPL</x:v>
       </x:c>
       <x:c r="J43" s="9" t="str">
-        <x:v>YES</x:v>
+        <x:v>NO</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="9" t="str">
-        <x:v>R17</x:v>
+        <x:v>R15</x:v>
       </x:c>
       <x:c r="B44" s="9" t="str">
-        <x:v>133k</x:v>
+        <x:v>100k</x:v>
       </x:c>
       <x:c r="C44" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1687,10 +1699,10 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" s="9" t="str">
-        <x:v>R18</x:v>
+        <x:v>R16</x:v>
       </x:c>
       <x:c r="B45" s="9" t="str">
-        <x:v>10k</x:v>
+        <x:v>33k2</x:v>
       </x:c>
       <x:c r="C45" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1715,10 +1727,10 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" s="9" t="str">
-        <x:v>R19</x:v>
+        <x:v>R17</x:v>
       </x:c>
       <x:c r="B46" s="9" t="str">
-        <x:v>0R</x:v>
+        <x:v>133k</x:v>
       </x:c>
       <x:c r="C46" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1743,10 +1755,10 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" s="9" t="str">
-        <x:v>R20</x:v>
+        <x:v>R18</x:v>
       </x:c>
       <x:c r="B47" s="9" t="str">
-        <x:v>470k</x:v>
+        <x:v>10k</x:v>
       </x:c>
       <x:c r="C47" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1771,10 +1783,10 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" s="9" t="str">
-        <x:v>R21</x:v>
+        <x:v>R19</x:v>
       </x:c>
       <x:c r="B48" s="9" t="str">
-        <x:v>100k</x:v>
+        <x:v>0R</x:v>
       </x:c>
       <x:c r="C48" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1799,10 +1811,10 @@
     </x:row>
     <x:row r="49">
       <x:c r="A49" s="9" t="str">
-        <x:v>R22</x:v>
+        <x:v>R20</x:v>
       </x:c>
       <x:c r="B49" s="9" t="str">
-        <x:v>101k</x:v>
+        <x:v>470k</x:v>
       </x:c>
       <x:c r="C49" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1827,10 +1839,10 @@
     </x:row>
     <x:row r="50">
       <x:c r="A50" s="9" t="str">
-        <x:v>R23</x:v>
+        <x:v>R21</x:v>
       </x:c>
       <x:c r="B50" s="9" t="str">
-        <x:v>10k</x:v>
+        <x:v>100k</x:v>
       </x:c>
       <x:c r="C50" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1855,10 +1867,10 @@
     </x:row>
     <x:row r="51">
       <x:c r="A51" s="9" t="str">
-        <x:v>R24</x:v>
+        <x:v>R22</x:v>
       </x:c>
       <x:c r="B51" s="9" t="str">
-        <x:v>100k</x:v>
+        <x:v>101k</x:v>
       </x:c>
       <x:c r="C51" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1883,10 +1895,10 @@
     </x:row>
     <x:row r="52">
       <x:c r="A52" s="9" t="str">
-        <x:v>R25</x:v>
+        <x:v>R23</x:v>
       </x:c>
       <x:c r="B52" s="9" t="str">
-        <x:v>12k</x:v>
+        <x:v>10k</x:v>
       </x:c>
       <x:c r="C52" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1911,10 +1923,10 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="9" t="str">
-        <x:v>R26</x:v>
+        <x:v>R24</x:v>
       </x:c>
       <x:c r="B53" s="9" t="str">
-        <x:v>820R</x:v>
+        <x:v>100k</x:v>
       </x:c>
       <x:c r="C53" s="9" t="str">
         <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
@@ -1939,31 +1951,27 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="9" t="str">
-        <x:v>U1</x:v>
+        <x:v>R25</x:v>
       </x:c>
       <x:c r="B54" s="9" t="str">
-        <x:v>STUSB4500QTR</x:v>
+        <x:v>12k</x:v>
       </x:c>
       <x:c r="C54" s="9" t="str">
-        <x:v>Package_DFN_QFN:QFN-24-1EP_4x4mm_P0.5mm_EP2.7x2.7mm</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D54" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E54" s="9" t="str">
-        <x:v>STUSB4500QTR</x:v>
-      </x:c>
-      <x:c r="F54" s="9" t="str">
-        <x:v>C2678061</x:v>
-      </x:c>
+      <x:c r="E54" s="9" t="str"/>
+      <x:c r="F54" s="9" t="str"/>
       <x:c r="G54" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H54" s="12" t="str">
-        <x:v>SKU CANDIDATE</x:v>
+        <x:v>SKU NOT ASSIGNED</x:v>
       </x:c>
       <x:c r="I54" s="9" t="str">
-        <x:v>STUSB4500 NVM programming required</x:v>
+        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
       </x:c>
       <x:c r="J54" s="9" t="str">
         <x:v>YES</x:v>
@@ -1971,54 +1979,50 @@
     </x:row>
     <x:row r="55">
       <x:c r="A55" s="9" t="str">
-        <x:v>U2</x:v>
+        <x:v>R26</x:v>
       </x:c>
       <x:c r="B55" s="9" t="str">
-        <x:v>LM61460AASQRJRRQ1</x:v>
+        <x:v>820R</x:v>
       </x:c>
       <x:c r="C55" s="9" t="str">
-        <x:v>FT2D:TI_RJR0014A</x:v>
+        <x:v>Resistor_SMD:R_0603_1608Metric</x:v>
       </x:c>
       <x:c r="D55" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E55" s="9" t="str">
-        <x:v>LM61460AASQRJRRQ1</x:v>
-      </x:c>
-      <x:c r="F55" s="9" t="str">
-        <x:v>C1855832</x:v>
-      </x:c>
+      <x:c r="E55" s="9" t="str"/>
+      <x:c r="F55" s="9" t="str"/>
       <x:c r="G55" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H55" s="12" t="str">
-        <x:v>SKU CANDIDATE</x:v>
+        <x:v>SKU NOT ASSIGNED</x:v>
       </x:c>
       <x:c r="I55" s="9" t="str">
-        <x:v>Verify custom RJR land pattern</x:v>
+        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
       </x:c>
       <x:c r="J55" s="9" t="str">
-        <x:v>NO</x:v>
+        <x:v>YES</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
       <x:c r="A56" s="9" t="str">
-        <x:v>U3</x:v>
+        <x:v>U1</x:v>
       </x:c>
       <x:c r="B56" s="9" t="str">
-        <x:v>TPS259474ARPWR</x:v>
+        <x:v>STUSB4500QTR</x:v>
       </x:c>
       <x:c r="C56" s="9" t="str">
-        <x:v>FT2D:TI_RPW0010A</x:v>
+        <x:v>Package_DFN_QFN:QFN-24-1EP_4x4mm_P0.5mm_EP2.7x2.7mm</x:v>
       </x:c>
       <x:c r="D56" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E56" s="9" t="str">
-        <x:v>TPS259474ARPWR</x:v>
+        <x:v>STUSB4500QTR</x:v>
       </x:c>
       <x:c r="F56" s="9" t="str">
-        <x:v>C3662807</x:v>
+        <x:v>C2678061</x:v>
       </x:c>
       <x:c r="G56" s="9" t="str">
         <x:v>SMT</x:v>
@@ -2027,10 +2031,74 @@
         <x:v>SKU CANDIDATE</x:v>
       </x:c>
       <x:c r="I56" s="9" t="str">
+        <x:v>STUSB4500 NVM programming required</x:v>
+      </x:c>
+      <x:c r="J56" s="9" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="9" t="str">
+        <x:v>U2</x:v>
+      </x:c>
+      <x:c r="B57" s="9" t="str">
+        <x:v>LM61460AASQRJRRQ1</x:v>
+      </x:c>
+      <x:c r="C57" s="9" t="str">
+        <x:v>FT2D:TI_RJR0014A</x:v>
+      </x:c>
+      <x:c r="D57" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E57" s="9" t="str">
+        <x:v>LM61460AASQRJRRQ1</x:v>
+      </x:c>
+      <x:c r="F57" s="9" t="str">
+        <x:v>C1855832</x:v>
+      </x:c>
+      <x:c r="G57" s="9" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="H57" s="12" t="str">
+        <x:v>SKU CANDIDATE</x:v>
+      </x:c>
+      <x:c r="I57" s="9" t="str">
+        <x:v>Verify custom RJR land pattern</x:v>
+      </x:c>
+      <x:c r="J57" s="9" t="str">
+        <x:v>YES</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="9" t="str">
+        <x:v>U3</x:v>
+      </x:c>
+      <x:c r="B58" s="9" t="str">
+        <x:v>TPS259474ARPWR</x:v>
+      </x:c>
+      <x:c r="C58" s="9" t="str">
+        <x:v>FT2D:TI_RPW0010A</x:v>
+      </x:c>
+      <x:c r="D58" s="10" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E58" s="9" t="str">
+        <x:v>TPS259474ARPWR</x:v>
+      </x:c>
+      <x:c r="F58" s="9" t="str">
+        <x:v>C3662807</x:v>
+      </x:c>
+      <x:c r="G58" s="9" t="str">
+        <x:v>SMT</x:v>
+      </x:c>
+      <x:c r="H58" s="12" t="str">
+        <x:v>SKU CANDIDATE</x:v>
+      </x:c>
+      <x:c r="I58" s="9" t="str">
         <x:v>Verify RPW land pattern and current limit</x:v>
       </x:c>
-      <x:c r="J56" s="9" t="str">
-        <x:v>NO</x:v>
+      <x:c r="J58" s="9" t="str">
+        <x:v>YES</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2092,16 +2160,16 @@
       <x:c r="C2" t="str">
         <x:v>C_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D2" s="15" t="n">
+      <x:c r="D2" s="17" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="E2" s="15" t="n">
+      <x:c r="E2" s="17" t="n">
         <x:v>-35</x:v>
       </x:c>
-      <x:c r="F2" s="15" t="n">
+      <x:c r="F2" s="17" t="n">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="G2" s="15" t="n">
+      <x:c r="G2" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H2" t="str">
@@ -2121,16 +2189,16 @@
       <x:c r="C3" t="str">
         <x:v>C_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D3" s="15" t="n">
+      <x:c r="D3" s="17" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="E3" s="15" t="n">
+      <x:c r="E3" s="17" t="n">
         <x:v>-35</x:v>
       </x:c>
-      <x:c r="F3" s="15" t="n">
+      <x:c r="F3" s="17" t="n">
         <x:v>35</x:v>
       </x:c>
-      <x:c r="G3" s="15" t="n">
+      <x:c r="G3" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H3" t="str">
@@ -2150,16 +2218,16 @@
       <x:c r="C4" t="str">
         <x:v>C_0805_2012Metric</x:v>
       </x:c>
-      <x:c r="D4" s="15" t="n">
+      <x:c r="D4" s="17" t="n">
         <x:v>50</x:v>
       </x:c>
-      <x:c r="E4" s="15" t="n">
+      <x:c r="E4" s="17" t="n">
         <x:v>-41</x:v>
       </x:c>
-      <x:c r="F4" s="15" t="n">
+      <x:c r="F4" s="17" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="G4" s="15" t="n">
+      <x:c r="G4" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H4" t="str">
@@ -2179,16 +2247,16 @@
       <x:c r="C5" t="str">
         <x:v>C_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D5" s="15" t="n">
+      <x:c r="D5" s="17" t="n">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="E5" s="15" t="n">
+      <x:c r="E5" s="17" t="n">
         <x:v>-56</x:v>
       </x:c>
-      <x:c r="F5" s="15" t="n">
+      <x:c r="F5" s="17" t="n">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="G5" s="15" t="n">
+      <x:c r="G5" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H5" t="str">
@@ -2208,16 +2276,16 @@
       <x:c r="C6" t="str">
         <x:v>C_0805_2012Metric</x:v>
       </x:c>
-      <x:c r="D6" s="15" t="n">
+      <x:c r="D6" s="17" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="E6" s="15" t="n">
+      <x:c r="E6" s="17" t="n">
         <x:v>-46</x:v>
       </x:c>
-      <x:c r="F6" s="15" t="n">
+      <x:c r="F6" s="17" t="n">
         <x:v>46</x:v>
       </x:c>
-      <x:c r="G6" s="15" t="n">
+      <x:c r="G6" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H6" t="str">
@@ -2237,16 +2305,16 @@
       <x:c r="C7" t="str">
         <x:v>C_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D7" s="15" t="n">
+      <x:c r="D7" s="17" t="n">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="E7" s="15" t="n">
+      <x:c r="E7" s="17" t="n">
         <x:v>-47</x:v>
       </x:c>
-      <x:c r="F7" s="15" t="n">
+      <x:c r="F7" s="17" t="n">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="G7" s="15" t="n">
+      <x:c r="G7" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H7" t="str">
@@ -2266,16 +2334,16 @@
       <x:c r="C8" t="str">
         <x:v>C_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D8" s="15" t="n">
-        <x:v>69</x:v>
-      </x:c>
-      <x:c r="E8" s="15" t="n">
+      <x:c r="D8" s="17" t="n">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="E8" s="17" t="n">
         <x:v>-38</x:v>
       </x:c>
-      <x:c r="F8" s="15" t="n">
+      <x:c r="F8" s="17" t="n">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="G8" s="15" t="n">
+      <x:c r="G8" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H8" t="str">
@@ -2295,16 +2363,16 @@
       <x:c r="C9" t="str">
         <x:v>C_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D9" s="15" t="n">
-        <x:v>75</x:v>
-      </x:c>
-      <x:c r="E9" s="15" t="n">
+      <x:c r="D9" s="17" t="n">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="E9" s="17" t="n">
         <x:v>-38</x:v>
       </x:c>
-      <x:c r="F9" s="15" t="n">
+      <x:c r="F9" s="17" t="n">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="G9" s="15" t="n">
+      <x:c r="G9" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H9" t="str">
@@ -2324,16 +2392,16 @@
       <x:c r="C10" t="str">
         <x:v>C_1210_3225Metric</x:v>
       </x:c>
-      <x:c r="D10" s="15" t="n">
+      <x:c r="D10" s="17" t="n">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="E10" s="15" t="n">
+      <x:c r="E10" s="17" t="n">
         <x:v>-33</x:v>
       </x:c>
-      <x:c r="F10" s="15" t="n">
+      <x:c r="F10" s="17" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="G10" s="15" t="n">
+      <x:c r="G10" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H10" t="str">
@@ -2353,16 +2421,16 @@
       <x:c r="C11" t="str">
         <x:v>C_1210_3225Metric</x:v>
       </x:c>
-      <x:c r="D11" s="15" t="n">
+      <x:c r="D11" s="17" t="n">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="E11" s="15" t="n">
+      <x:c r="E11" s="17" t="n">
         <x:v>-33</x:v>
       </x:c>
-      <x:c r="F11" s="15" t="n">
+      <x:c r="F11" s="17" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="G11" s="15" t="n">
+      <x:c r="G11" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H11" t="str">
@@ -2382,16 +2450,16 @@
       <x:c r="C12" t="str">
         <x:v>C_1210_3225Metric</x:v>
       </x:c>
-      <x:c r="D12" s="15" t="n">
+      <x:c r="D12" s="17" t="n">
         <x:v>72</x:v>
       </x:c>
-      <x:c r="E12" s="15" t="n">
+      <x:c r="E12" s="17" t="n">
         <x:v>-33</x:v>
       </x:c>
-      <x:c r="F12" s="15" t="n">
+      <x:c r="F12" s="17" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="G12" s="15" t="n">
+      <x:c r="G12" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H12" t="str">
@@ -2411,16 +2479,16 @@
       <x:c r="C13" t="str">
         <x:v>C_1210_3225Metric</x:v>
       </x:c>
-      <x:c r="D13" s="15" t="n">
+      <x:c r="D13" s="17" t="n">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="E13" s="15" t="n">
+      <x:c r="E13" s="17" t="n">
         <x:v>-33</x:v>
       </x:c>
-      <x:c r="F13" s="15" t="n">
+      <x:c r="F13" s="17" t="n">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="G13" s="15" t="n">
+      <x:c r="G13" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H13" t="str">
@@ -2440,16 +2508,16 @@
       <x:c r="C14" t="str">
         <x:v>CP_Elec_5x5.8</x:v>
       </x:c>
-      <x:c r="D14" s="15" t="n">
+      <x:c r="D14" s="17" t="n">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="E14" s="15" t="n">
+      <x:c r="E14" s="17" t="n">
         <x:v>-48</x:v>
       </x:c>
-      <x:c r="F14" s="15" t="n">
+      <x:c r="F14" s="17" t="n">
         <x:v>48</x:v>
       </x:c>
-      <x:c r="G14" s="15" t="n">
+      <x:c r="G14" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H14" t="str">
@@ -2469,16 +2537,16 @@
       <x:c r="C15" t="str">
         <x:v>C_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D15" s="15" t="n">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="E15" s="15" t="n">
-        <x:v>-45</x:v>
-      </x:c>
-      <x:c r="F15" s="15" t="n">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="G15" s="15" t="n">
+      <x:c r="D15" s="17" t="n">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="E15" s="17" t="n">
+        <x:v>-48.5</x:v>
+      </x:c>
+      <x:c r="F15" s="17" t="n">
+        <x:v>48.5</x:v>
+      </x:c>
+      <x:c r="G15" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H15" t="str">
@@ -2498,16 +2566,16 @@
       <x:c r="C16" t="str">
         <x:v>C_1210_3225Metric</x:v>
       </x:c>
-      <x:c r="D16" s="15" t="n">
+      <x:c r="D16" s="17" t="n">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="E16" s="15" t="n">
+      <x:c r="E16" s="17" t="n">
         <x:v>-34</x:v>
       </x:c>
-      <x:c r="F16" s="15" t="n">
+      <x:c r="F16" s="17" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="G16" s="15" t="n">
+      <x:c r="G16" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H16" t="str">
@@ -2527,16 +2595,16 @@
       <x:c r="C17" t="str">
         <x:v>C_1210_3225Metric</x:v>
       </x:c>
-      <x:c r="D17" s="15" t="n">
+      <x:c r="D17" s="17" t="n">
         <x:v>103</x:v>
       </x:c>
-      <x:c r="E17" s="15" t="n">
+      <x:c r="E17" s="17" t="n">
         <x:v>-34</x:v>
       </x:c>
-      <x:c r="F17" s="15" t="n">
+      <x:c r="F17" s="17" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="G17" s="15" t="n">
+      <x:c r="G17" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H17" t="str">
@@ -2556,16 +2624,16 @@
       <x:c r="C18" t="str">
         <x:v>C_1210_3225Metric</x:v>
       </x:c>
-      <x:c r="D18" s="15" t="n">
+      <x:c r="D18" s="17" t="n">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="E18" s="15" t="n">
+      <x:c r="E18" s="17" t="n">
         <x:v>-34</x:v>
       </x:c>
-      <x:c r="F18" s="15" t="n">
+      <x:c r="F18" s="17" t="n">
         <x:v>34</x:v>
       </x:c>
-      <x:c r="G18" s="15" t="n">
+      <x:c r="G18" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H18" t="str">
@@ -2585,16 +2653,16 @@
       <x:c r="C19" t="str">
         <x:v>CP_Elec_6.3x7.7</x:v>
       </x:c>
-      <x:c r="D19" s="15" t="n">
+      <x:c r="D19" s="17" t="n">
         <x:v>102</x:v>
       </x:c>
-      <x:c r="E19" s="15" t="n">
+      <x:c r="E19" s="17" t="n">
         <x:v>-51</x:v>
       </x:c>
-      <x:c r="F19" s="15" t="n">
+      <x:c r="F19" s="17" t="n">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="G19" s="15" t="n">
+      <x:c r="G19" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H19" t="str">
@@ -2614,16 +2682,16 @@
       <x:c r="C20" t="str">
         <x:v>C_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D20" s="15" t="n">
+      <x:c r="D20" s="17" t="n">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="E20" s="15" t="n">
+      <x:c r="E20" s="17" t="n">
         <x:v>-41</x:v>
       </x:c>
-      <x:c r="F20" s="15" t="n">
+      <x:c r="F20" s="17" t="n">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="G20" s="15" t="n">
+      <x:c r="G20" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H20" t="str">
@@ -2643,16 +2711,16 @@
       <x:c r="C21" t="str">
         <x:v>C_1210_3225Metric</x:v>
       </x:c>
-      <x:c r="D21" s="15" t="n">
+      <x:c r="D21" s="17" t="n">
         <x:v>117</x:v>
       </x:c>
-      <x:c r="E21" s="15" t="n">
+      <x:c r="E21" s="17" t="n">
         <x:v>-51</x:v>
       </x:c>
-      <x:c r="F21" s="15" t="n">
+      <x:c r="F21" s="17" t="n">
         <x:v>51</x:v>
       </x:c>
-      <x:c r="G21" s="15" t="n">
+      <x:c r="G21" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H21" t="str">
@@ -2672,16 +2740,16 @@
       <x:c r="C22" t="str">
         <x:v>C_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D22" s="15" t="n">
+      <x:c r="D22" s="17" t="n">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="E22" s="15" t="n">
+      <x:c r="E22" s="17" t="n">
         <x:v>-43</x:v>
       </x:c>
-      <x:c r="F22" s="15" t="n">
+      <x:c r="F22" s="17" t="n">
         <x:v>43</x:v>
       </x:c>
-      <x:c r="G22" s="15" t="n">
+      <x:c r="G22" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H22" t="str">
@@ -2701,16 +2769,16 @@
       <x:c r="C23" t="str">
         <x:v>C_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D23" s="15" t="n">
+      <x:c r="D23" s="17" t="n">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="E23" s="15" t="n">
+      <x:c r="E23" s="17" t="n">
         <x:v>-49</x:v>
       </x:c>
-      <x:c r="F23" s="15" t="n">
+      <x:c r="F23" s="17" t="n">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="G23" s="15" t="n">
+      <x:c r="G23" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H23" t="str">
@@ -2730,16 +2798,16 @@
       <x:c r="C24" t="str">
         <x:v>C_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D24" s="15" t="n">
+      <x:c r="D24" s="17" t="n">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="E24" s="15" t="n">
+      <x:c r="E24" s="17" t="n">
         <x:v>-49</x:v>
       </x:c>
-      <x:c r="F24" s="15" t="n">
+      <x:c r="F24" s="17" t="n">
         <x:v>49</x:v>
       </x:c>
-      <x:c r="G24" s="15" t="n">
+      <x:c r="G24" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H24" t="str">
@@ -2751,24 +2819,24 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
-        <x:v>D2</x:v>
+        <x:v>D1</x:v>
       </x:c>
       <x:c r="B25" t="str">
-        <x:v>ESDA25W</x:v>
+        <x:v>ESDA25P35-1U1M</x:v>
       </x:c>
       <x:c r="C25" t="str">
-        <x:v>SOT-323_SC-70</x:v>
-      </x:c>
-      <x:c r="D25" s="15" t="n">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="E25" s="15" t="n">
-        <x:v>-37</x:v>
-      </x:c>
-      <x:c r="F25" s="15" t="n">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="G25" s="15" t="n">
+        <x:v>ST_ESDA25P35_1U1M</x:v>
+      </x:c>
+      <x:c r="D25" s="17" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="E25" s="17" t="n">
+        <x:v>-46</x:v>
+      </x:c>
+      <x:c r="F25" s="17" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="G25" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H25" t="str">
@@ -2780,24 +2848,24 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="str">
-        <x:v>F1</x:v>
+        <x:v>D2</x:v>
       </x:c>
       <x:c r="B26" t="str">
-        <x:v>1206SFS300F/32</x:v>
+        <x:v>ESDA25W</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>Fuse_1206_3216Metric</x:v>
-      </x:c>
-      <x:c r="D26" s="15" t="n">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="E26" s="15" t="n">
-        <x:v>-43</x:v>
-      </x:c>
-      <x:c r="F26" s="15" t="n">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="G26" s="15" t="n">
+        <x:v>SOT-323_SC-70</x:v>
+      </x:c>
+      <x:c r="D26" s="17" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="E26" s="17" t="n">
+        <x:v>-37</x:v>
+      </x:c>
+      <x:c r="F26" s="17" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="G26" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H26" t="str">
@@ -2809,24 +2877,24 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" t="str">
-        <x:v>R1</x:v>
+        <x:v>F1</x:v>
       </x:c>
       <x:c r="B27" t="str">
-        <x:v>10k</x:v>
+        <x:v>1206SFS300F/32</x:v>
       </x:c>
       <x:c r="C27" t="str">
-        <x:v>R_0603_1608Metric</x:v>
-      </x:c>
-      <x:c r="D27" s="15" t="n">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="E27" s="15" t="n">
-        <x:v>-51</x:v>
-      </x:c>
-      <x:c r="F27" s="15" t="n">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="G27" s="15" t="n">
+        <x:v>Fuse_1206_3216Metric</x:v>
+      </x:c>
+      <x:c r="D27" s="17" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="E27" s="17" t="n">
+        <x:v>-43</x:v>
+      </x:c>
+      <x:c r="F27" s="17" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="G27" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H27" t="str">
@@ -2838,25 +2906,25 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" t="str">
-        <x:v>R2</x:v>
+        <x:v>J1</x:v>
       </x:c>
       <x:c r="B28" t="str">
-        <x:v>4k7</x:v>
+        <x:v>TYPE-C-31-M-12</x:v>
       </x:c>
       <x:c r="C28" t="str">
-        <x:v>R_0603_1608Metric</x:v>
-      </x:c>
-      <x:c r="D28" s="15" t="n">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="E28" s="15" t="n">
-        <x:v>-51</x:v>
-      </x:c>
-      <x:c r="F28" s="15" t="n">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="G28" s="15" t="n">
-        <x:v>0</x:v>
+        <x:v>USB_C_Receptacle_HRO_TYPE-C-31-M-12</x:v>
+      </x:c>
+      <x:c r="D28" s="17" t="n">
+        <x:v>24.15</x:v>
+      </x:c>
+      <x:c r="E28" s="17" t="n">
+        <x:v>-42</x:v>
+      </x:c>
+      <x:c r="F28" s="17" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="G28" s="17" t="n">
+        <x:v>-90</x:v>
       </x:c>
       <x:c r="H28" t="str">
         <x:v>top</x:v>
@@ -2867,24 +2935,24 @@
     </x:row>
     <x:row r="29">
       <x:c r="A29" t="str">
-        <x:v>R3</x:v>
+        <x:v>L1</x:v>
       </x:c>
       <x:c r="B29" t="str">
-        <x:v>4k7</x:v>
+        <x:v>SRG1260-100-M_10uH</x:v>
       </x:c>
       <x:c r="C29" t="str">
-        <x:v>R_0603_1608Metric</x:v>
-      </x:c>
-      <x:c r="D29" s="15" t="n">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="E29" s="15" t="n">
-        <x:v>-51</x:v>
-      </x:c>
-      <x:c r="F29" s="15" t="n">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="G29" s="15" t="n">
+        <x:v>JIERR_SRG1260_100M</x:v>
+      </x:c>
+      <x:c r="D29" s="17" t="n">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="E29" s="17" t="n">
+        <x:v>-43</x:v>
+      </x:c>
+      <x:c r="F29" s="17" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="G29" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H29" t="str">
@@ -2896,24 +2964,24 @@
     </x:row>
     <x:row r="30">
       <x:c r="A30" t="str">
-        <x:v>R4</x:v>
+        <x:v>Q1</x:v>
       </x:c>
       <x:c r="B30" t="str">
-        <x:v>1k</x:v>
+        <x:v>STL6P3LLH6</x:v>
       </x:c>
       <x:c r="C30" t="str">
-        <x:v>R_0603_1608Metric</x:v>
-      </x:c>
-      <x:c r="D30" s="15" t="n">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E30" s="15" t="n">
-        <x:v>-47</x:v>
-      </x:c>
-      <x:c r="F30" s="15" t="n">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="G30" s="15" t="n">
+        <x:v>ST_PowerFLAT_3p3_TypeF</x:v>
+      </x:c>
+      <x:c r="D30" s="17" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="E30" s="17" t="n">
+        <x:v>-42</x:v>
+      </x:c>
+      <x:c r="F30" s="17" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="G30" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H30" t="str">
@@ -2925,24 +2993,24 @@
     </x:row>
     <x:row r="31">
       <x:c r="A31" t="str">
-        <x:v>R5</x:v>
+        <x:v>R1</x:v>
       </x:c>
       <x:c r="B31" t="str">
-        <x:v>22k</x:v>
+        <x:v>10k</x:v>
       </x:c>
       <x:c r="C31" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D31" s="15" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="E31" s="15" t="n">
-        <x:v>-52</x:v>
-      </x:c>
-      <x:c r="F31" s="15" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="G31" s="15" t="n">
+      <x:c r="D31" s="17" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="E31" s="17" t="n">
+        <x:v>-51</x:v>
+      </x:c>
+      <x:c r="F31" s="17" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G31" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H31" t="str">
@@ -2954,24 +3022,24 @@
     </x:row>
     <x:row r="32">
       <x:c r="A32" t="str">
-        <x:v>R6</x:v>
+        <x:v>R2</x:v>
       </x:c>
       <x:c r="B32" t="str">
-        <x:v>470R</x:v>
+        <x:v>4k7</x:v>
       </x:c>
       <x:c r="C32" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D32" s="15" t="n">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="E32" s="15" t="n">
-        <x:v>-50</x:v>
-      </x:c>
-      <x:c r="F32" s="15" t="n">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="G32" s="15" t="n">
+      <x:c r="D32" s="17" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="E32" s="17" t="n">
+        <x:v>-51</x:v>
+      </x:c>
+      <x:c r="F32" s="17" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G32" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H32" t="str">
@@ -2983,24 +3051,24 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" t="str">
-        <x:v>R7</x:v>
+        <x:v>R3</x:v>
       </x:c>
       <x:c r="B33" t="str">
-        <x:v>100k</x:v>
+        <x:v>4k7</x:v>
       </x:c>
       <x:c r="C33" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D33" s="15" t="n">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="E33" s="15" t="n">
-        <x:v>-52</x:v>
-      </x:c>
-      <x:c r="F33" s="15" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="G33" s="15" t="n">
+      <x:c r="D33" s="17" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="E33" s="17" t="n">
+        <x:v>-51</x:v>
+      </x:c>
+      <x:c r="F33" s="17" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G33" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H33" t="str">
@@ -3012,24 +3080,24 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" t="str">
-        <x:v>R12</x:v>
+        <x:v>R4</x:v>
       </x:c>
       <x:c r="B34" t="str">
-        <x:v>100k_0.1%</x:v>
+        <x:v>1k</x:v>
       </x:c>
       <x:c r="C34" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D34" s="15" t="n">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="E34" s="15" t="n">
-        <x:v>-52</x:v>
-      </x:c>
-      <x:c r="F34" s="15" t="n">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="G34" s="15" t="n">
+      <x:c r="D34" s="17" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E34" s="17" t="n">
+        <x:v>-47</x:v>
+      </x:c>
+      <x:c r="F34" s="17" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="G34" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H34" t="str">
@@ -3041,24 +3109,24 @@
     </x:row>
     <x:row r="35">
       <x:c r="A35" t="str">
-        <x:v>R13</x:v>
+        <x:v>R5</x:v>
       </x:c>
       <x:c r="B35" t="str">
-        <x:v>8k66_0.1%</x:v>
+        <x:v>22k</x:v>
       </x:c>
       <x:c r="C35" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D35" s="15" t="n">
-        <x:v>78</x:v>
-      </x:c>
-      <x:c r="E35" s="15" t="n">
-        <x:v>-55</x:v>
-      </x:c>
-      <x:c r="F35" s="15" t="n">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="G35" s="15" t="n">
+      <x:c r="D35" s="17" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E35" s="17" t="n">
+        <x:v>-52</x:v>
+      </x:c>
+      <x:c r="F35" s="17" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="G35" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H35" t="str">
@@ -3070,24 +3138,24 @@
     </x:row>
     <x:row r="36">
       <x:c r="A36" t="str">
-        <x:v>R15</x:v>
+        <x:v>R6</x:v>
       </x:c>
       <x:c r="B36" t="str">
-        <x:v>100k</x:v>
+        <x:v>470R</x:v>
       </x:c>
       <x:c r="C36" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D36" s="15" t="n">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="E36" s="15" t="n">
-        <x:v>-51</x:v>
-      </x:c>
-      <x:c r="F36" s="15" t="n">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="G36" s="15" t="n">
+      <x:c r="D36" s="17" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="E36" s="17" t="n">
+        <x:v>-50</x:v>
+      </x:c>
+      <x:c r="F36" s="17" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G36" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H36" t="str">
@@ -3099,24 +3167,24 @@
     </x:row>
     <x:row r="37">
       <x:c r="A37" t="str">
-        <x:v>R16</x:v>
+        <x:v>R7</x:v>
       </x:c>
       <x:c r="B37" t="str">
-        <x:v>33k2</x:v>
+        <x:v>100k</x:v>
       </x:c>
       <x:c r="C37" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D37" s="15" t="n">
-        <x:v>71</x:v>
-      </x:c>
-      <x:c r="E37" s="15" t="n">
-        <x:v>-51</x:v>
-      </x:c>
-      <x:c r="F37" s="15" t="n">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="G37" s="15" t="n">
+      <x:c r="D37" s="17" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="E37" s="17" t="n">
+        <x:v>-52</x:v>
+      </x:c>
+      <x:c r="F37" s="17" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="G37" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H37" t="str">
@@ -3128,24 +3196,24 @@
     </x:row>
     <x:row r="38">
       <x:c r="A38" t="str">
-        <x:v>R17</x:v>
+        <x:v>R12</x:v>
       </x:c>
       <x:c r="B38" t="str">
-        <x:v>133k</x:v>
+        <x:v>100k_0.1%</x:v>
       </x:c>
       <x:c r="C38" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D38" s="15" t="n">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="E38" s="15" t="n">
-        <x:v>-55</x:v>
-      </x:c>
-      <x:c r="F38" s="15" t="n">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="G38" s="15" t="n">
+      <x:c r="D38" s="17" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="E38" s="17" t="n">
+        <x:v>-52</x:v>
+      </x:c>
+      <x:c r="F38" s="17" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="G38" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H38" t="str">
@@ -3157,24 +3225,24 @@
     </x:row>
     <x:row r="39">
       <x:c r="A39" t="str">
-        <x:v>R18</x:v>
+        <x:v>R13</x:v>
       </x:c>
       <x:c r="B39" t="str">
-        <x:v>10k</x:v>
+        <x:v>8k66_0.1%</x:v>
       </x:c>
       <x:c r="C39" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D39" s="15" t="n">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="E39" s="15" t="n">
+      <x:c r="D39" s="17" t="n">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="E39" s="17" t="n">
         <x:v>-55</x:v>
       </x:c>
-      <x:c r="F39" s="15" t="n">
+      <x:c r="F39" s="17" t="n">
         <x:v>55</x:v>
       </x:c>
-      <x:c r="G39" s="15" t="n">
+      <x:c r="G39" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H39" t="str">
@@ -3186,24 +3254,24 @@
     </x:row>
     <x:row r="40">
       <x:c r="A40" t="str">
-        <x:v>R19</x:v>
+        <x:v>R15</x:v>
       </x:c>
       <x:c r="B40" t="str">
-        <x:v>0R</x:v>
+        <x:v>100k</x:v>
       </x:c>
       <x:c r="C40" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D40" s="15" t="n">
-        <x:v>77</x:v>
-      </x:c>
-      <x:c r="E40" s="15" t="n">
-        <x:v>-48</x:v>
-      </x:c>
-      <x:c r="F40" s="15" t="n">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="G40" s="15" t="n">
+      <x:c r="D40" s="17" t="n">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="E40" s="17" t="n">
+        <x:v>-51</x:v>
+      </x:c>
+      <x:c r="F40" s="17" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G40" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H40" t="str">
@@ -3215,24 +3283,24 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" t="str">
-        <x:v>R20</x:v>
+        <x:v>R16</x:v>
       </x:c>
       <x:c r="B41" t="str">
-        <x:v>470k</x:v>
+        <x:v>33k2</x:v>
       </x:c>
       <x:c r="C41" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D41" s="15" t="n">
-        <x:v>114</x:v>
-      </x:c>
-      <x:c r="E41" s="15" t="n">
-        <x:v>-60</x:v>
-      </x:c>
-      <x:c r="F41" s="15" t="n">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="G41" s="15" t="n">
+      <x:c r="D41" s="17" t="n">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="E41" s="17" t="n">
+        <x:v>-51</x:v>
+      </x:c>
+      <x:c r="F41" s="17" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="G41" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H41" t="str">
@@ -3244,24 +3312,24 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" t="str">
-        <x:v>R21</x:v>
+        <x:v>R17</x:v>
       </x:c>
       <x:c r="B42" t="str">
-        <x:v>100k</x:v>
+        <x:v>133k</x:v>
       </x:c>
       <x:c r="C42" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D42" s="15" t="n">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="E42" s="15" t="n">
-        <x:v>-60</x:v>
-      </x:c>
-      <x:c r="F42" s="15" t="n">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="G42" s="15" t="n">
+      <x:c r="D42" s="17" t="n">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="E42" s="17" t="n">
+        <x:v>-55</x:v>
+      </x:c>
+      <x:c r="F42" s="17" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="G42" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H42" t="str">
@@ -3273,24 +3341,24 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" t="str">
-        <x:v>R22</x:v>
+        <x:v>R18</x:v>
       </x:c>
       <x:c r="B43" t="str">
-        <x:v>101k</x:v>
+        <x:v>10k</x:v>
       </x:c>
       <x:c r="C43" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D43" s="15" t="n">
-        <x:v>100</x:v>
-      </x:c>
-      <x:c r="E43" s="15" t="n">
-        <x:v>-46</x:v>
-      </x:c>
-      <x:c r="F43" s="15" t="n">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="G43" s="15" t="n">
+      <x:c r="D43" s="17" t="n">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="E43" s="17" t="n">
+        <x:v>-55</x:v>
+      </x:c>
+      <x:c r="F43" s="17" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="G43" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H43" t="str">
@@ -3302,24 +3370,24 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" t="str">
-        <x:v>R23</x:v>
+        <x:v>R19</x:v>
       </x:c>
       <x:c r="B44" t="str">
-        <x:v>10k</x:v>
+        <x:v>0R</x:v>
       </x:c>
       <x:c r="C44" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D44" s="15" t="n">
-        <x:v>111</x:v>
-      </x:c>
-      <x:c r="E44" s="15" t="n">
-        <x:v>-56</x:v>
-      </x:c>
-      <x:c r="F44" s="15" t="n">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="G44" s="15" t="n">
+      <x:c r="D44" s="17" t="n">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="E44" s="17" t="n">
+        <x:v>-48</x:v>
+      </x:c>
+      <x:c r="F44" s="17" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G44" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H44" t="str">
@@ -3331,24 +3399,24 @@
     </x:row>
     <x:row r="45">
       <x:c r="A45" t="str">
-        <x:v>R24</x:v>
+        <x:v>R20</x:v>
       </x:c>
       <x:c r="B45" t="str">
-        <x:v>100k</x:v>
+        <x:v>470k</x:v>
       </x:c>
       <x:c r="C45" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D45" s="15" t="n">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="E45" s="15" t="n">
-        <x:v>-59</x:v>
-      </x:c>
-      <x:c r="F45" s="15" t="n">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="G45" s="15" t="n">
+      <x:c r="D45" s="17" t="n">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="E45" s="17" t="n">
+        <x:v>-60</x:v>
+      </x:c>
+      <x:c r="F45" s="17" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G45" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H45" t="str">
@@ -3360,24 +3428,24 @@
     </x:row>
     <x:row r="46">
       <x:c r="A46" t="str">
-        <x:v>R25</x:v>
+        <x:v>R21</x:v>
       </x:c>
       <x:c r="B46" t="str">
-        <x:v>12k</x:v>
+        <x:v>100k</x:v>
       </x:c>
       <x:c r="C46" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D46" s="15" t="n">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="E46" s="15" t="n">
-        <x:v>-59</x:v>
-      </x:c>
-      <x:c r="F46" s="15" t="n">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="G46" s="15" t="n">
+      <x:c r="D46" s="17" t="n">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="E46" s="17" t="n">
+        <x:v>-60</x:v>
+      </x:c>
+      <x:c r="F46" s="17" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="G46" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H46" t="str">
@@ -3389,24 +3457,24 @@
     </x:row>
     <x:row r="47">
       <x:c r="A47" t="str">
-        <x:v>R26</x:v>
+        <x:v>R22</x:v>
       </x:c>
       <x:c r="B47" t="str">
-        <x:v>820R</x:v>
+        <x:v>101k</x:v>
       </x:c>
       <x:c r="C47" t="str">
         <x:v>R_0603_1608Metric</x:v>
       </x:c>
-      <x:c r="D47" s="15" t="n">
-        <x:v>108</x:v>
-      </x:c>
-      <x:c r="E47" s="15" t="n">
-        <x:v>-59</x:v>
-      </x:c>
-      <x:c r="F47" s="15" t="n">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="G47" s="15" t="n">
+      <x:c r="D47" s="17" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="E47" s="17" t="n">
+        <x:v>-46</x:v>
+      </x:c>
+      <x:c r="F47" s="17" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="G47" s="17" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="H47" t="str">
@@ -3418,30 +3486,204 @@
     </x:row>
     <x:row r="48">
       <x:c r="A48" t="str">
+        <x:v>R23</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>10k</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>R_0603_1608Metric</x:v>
+      </x:c>
+      <x:c r="D48" s="17" t="n">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="E48" s="17" t="n">
+        <x:v>-56</x:v>
+      </x:c>
+      <x:c r="F48" s="17" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="G48" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H48" t="str">
+        <x:v>top</x:v>
+      </x:c>
+      <x:c r="I48" s="12" t="str">
+        <x:v>CHECK orientation / center</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>R24</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>100k</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>R_0603_1608Metric</x:v>
+      </x:c>
+      <x:c r="D49" s="17" t="n">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="E49" s="17" t="n">
+        <x:v>-59</x:v>
+      </x:c>
+      <x:c r="F49" s="17" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="G49" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H49" t="str">
+        <x:v>top</x:v>
+      </x:c>
+      <x:c r="I49" s="12" t="str">
+        <x:v>CHECK orientation / center</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>R25</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>12k</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>R_0603_1608Metric</x:v>
+      </x:c>
+      <x:c r="D50" s="17" t="n">
+        <x:v>105</x:v>
+      </x:c>
+      <x:c r="E50" s="17" t="n">
+        <x:v>-59</x:v>
+      </x:c>
+      <x:c r="F50" s="17" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="G50" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H50" t="str">
+        <x:v>top</x:v>
+      </x:c>
+      <x:c r="I50" s="12" t="str">
+        <x:v>CHECK orientation / center</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>R26</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>820R</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>R_0603_1608Metric</x:v>
+      </x:c>
+      <x:c r="D51" s="17" t="n">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="E51" s="17" t="n">
+        <x:v>-59</x:v>
+      </x:c>
+      <x:c r="F51" s="17" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="G51" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>top</x:v>
+      </x:c>
+      <x:c r="I51" s="12" t="str">
+        <x:v>CHECK orientation / center</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
         <x:v>U1</x:v>
       </x:c>
-      <x:c r="B48" t="str">
+      <x:c r="B52" t="str">
         <x:v>STUSB4500QTR</x:v>
       </x:c>
-      <x:c r="C48" t="str">
+      <x:c r="C52" t="str">
         <x:v>QFN-24-1EP_4x4mm_P0.5mm_EP2.7x2.7mm</x:v>
       </x:c>
-      <x:c r="D48" s="15" t="n">
+      <x:c r="D52" s="17" t="n">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="E48" s="15" t="n">
+      <x:c r="E52" s="17" t="n">
         <x:v>-40</x:v>
       </x:c>
-      <x:c r="F48" s="15" t="n">
+      <x:c r="F52" s="17" t="n">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="G48" s="15" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H48" t="str">
-        <x:v>top</x:v>
-      </x:c>
-      <x:c r="I48" s="12" t="str">
+      <x:c r="G52" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H52" t="str">
+        <x:v>top</x:v>
+      </x:c>
+      <x:c r="I52" s="12" t="str">
+        <x:v>CHECK orientation / center</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" t="str">
+        <x:v>U2</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>LM61460AASQRJRRQ1</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>TI_RJR0014A</x:v>
+      </x:c>
+      <x:c r="D53" s="17" t="n">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="E53" s="17" t="n">
+        <x:v>-43</x:v>
+      </x:c>
+      <x:c r="F53" s="17" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="G53" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H53" t="str">
+        <x:v>top</x:v>
+      </x:c>
+      <x:c r="I53" s="12" t="str">
+        <x:v>CHECK orientation / center</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" t="str">
+        <x:v>U3</x:v>
+      </x:c>
+      <x:c r="B54" t="str">
+        <x:v>TPS259474ARPWR</x:v>
+      </x:c>
+      <x:c r="C54" t="str">
+        <x:v>TI_RPW0010A</x:v>
+      </x:c>
+      <x:c r="D54" s="17" t="n">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="E54" s="17" t="n">
+        <x:v>-43</x:v>
+      </x:c>
+      <x:c r="F54" s="17" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="G54" s="17" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H54" t="str">
+        <x:v>top</x:v>
+      </x:c>
+      <x:c r="I54" s="12" t="str">
         <x:v>CHECK orientation / center</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Rev B: clear ERC/DRC/GND, validate C18 JLC hybrid footprint, export QA Gerbers and SMT sourcing review (NO-GO)
</commit_message>
<xml_diff>
--- a/manufacturing/Rev_B/REVIEW_ONLY_NOT_FOR_FAB/FT2D_RevB_SMT_sourcing_DRAFT.xlsx
+++ b/manufacturing/Rev_B/REVIEW_ONLY_NOT_FOR_FAB/FT2D_RevB_SMT_sourcing_DRAFT.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="R78b72b3de5e84521"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM review" sheetId="2" r:id="R77e2722ba1ff463f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPL preview" sheetId="3" r:id="R72f6cb30431a4032"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="R4212f2852f1f4ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM review" sheetId="2" r:id="R038f215f37004454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPL preview" sheetId="3" r:id="R3c5e969274e64cce"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -378,7 +378,7 @@
         <x:v>PCB DRC</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>0 violations; 5 unconnected GND items (NO-GO)</x:v>
+        <x:v>0 violations; 0 unconnected; schematic parity 0 (KiCad 10.0.7)</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -394,15 +394,15 @@
         <x:v>JLCPCB sourcing</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
-        <x:v>Partial SKU matches only; stock unverified</x:v>
+        <x:v>Candidate C-codes for critical/R-C parts; most passives not sourced; stock unverified</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="7" t="str">
-        <x:v>J1 / L1</x:v>
+        <x:v>J1 / L1 / C18</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
-        <x:v>HRO C165948 and JIERR C53463013 selected; OEM pad dimensions checked</x:v>
+        <x:v>HRO C165948 / JIERR C53463013 / Panasonic C178639 (thermal review)</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -417,6 +417,7 @@
       <x:c r="A14" s="8" t="str">
         <x:v>For planning/preview only: this is NOT a release BOM/CPL.</x:v>
       </x:c>
+      <x:c r="B14"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -736,16 +737,20 @@
       <x:c r="D11" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E11" s="9" t="str"/>
-      <x:c r="F11" s="9" t="str"/>
+      <x:c r="E11" s="9" t="str">
+        <x:v>GRM32ER71H106KA12L</x:v>
+      </x:c>
+      <x:c r="F11" s="9" t="str">
+        <x:v>C77102</x:v>
+      </x:c>
       <x:c r="G11" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H11" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / DC BIAS REVIEW</x:v>
       </x:c>
       <x:c r="I11" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Murata X7R 10uF 50V 1210; measure effective µF at 20V &amp; stock</x:v>
       </x:c>
       <x:c r="J11" s="9" t="str">
         <x:v>YES</x:v>
@@ -764,16 +769,20 @@
       <x:c r="D12" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E12" s="9" t="str"/>
-      <x:c r="F12" s="9" t="str"/>
+      <x:c r="E12" s="9" t="str">
+        <x:v>GRM32ER71H106KA12L</x:v>
+      </x:c>
+      <x:c r="F12" s="9" t="str">
+        <x:v>C77102</x:v>
+      </x:c>
       <x:c r="G12" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H12" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / DC BIAS REVIEW</x:v>
       </x:c>
       <x:c r="I12" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Murata X7R 10uF 50V 1210; measure effective µF at 20V &amp; stock</x:v>
       </x:c>
       <x:c r="J12" s="9" t="str">
         <x:v>YES</x:v>
@@ -792,16 +801,20 @@
       <x:c r="D13" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E13" s="9" t="str"/>
-      <x:c r="F13" s="9" t="str"/>
+      <x:c r="E13" s="9" t="str">
+        <x:v>GRM32ER71H106KA12L</x:v>
+      </x:c>
+      <x:c r="F13" s="9" t="str">
+        <x:v>C77102</x:v>
+      </x:c>
       <x:c r="G13" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H13" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / DC BIAS REVIEW</x:v>
       </x:c>
       <x:c r="I13" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Murata X7R 10uF 50V 1210; measure effective µF at 20V &amp; stock</x:v>
       </x:c>
       <x:c r="J13" s="9" t="str">
         <x:v>YES</x:v>
@@ -820,16 +833,20 @@
       <x:c r="D14" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E14" s="9" t="str"/>
-      <x:c r="F14" s="9" t="str"/>
+      <x:c r="E14" s="9" t="str">
+        <x:v>GRM32ER71H106KA12L</x:v>
+      </x:c>
+      <x:c r="F14" s="9" t="str">
+        <x:v>C77102</x:v>
+      </x:c>
       <x:c r="G14" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H14" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / DC BIAS REVIEW</x:v>
       </x:c>
       <x:c r="I14" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Murata X7R 10uF 50V 1210; measure effective µF at 20V &amp; stock</x:v>
       </x:c>
       <x:c r="J14" s="9" t="str">
         <x:v>YES</x:v>
@@ -840,26 +857,28 @@
         <x:v>C18</x:v>
       </x:c>
       <x:c r="B15" s="9" t="str">
-        <x:v>EEHZL1V470R_47u</x:v>
+        <x:v>EEHZA1V470P_47u</x:v>
       </x:c>
       <x:c r="C15" s="9" t="str">
-        <x:v>Capacitor_SMD:CP_Elec_5x5.8</x:v>
+        <x:v>Capacitor_SMD:CP_Elec_6.3x5.8</x:v>
       </x:c>
       <x:c r="D15" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="E15" s="9" t="str">
-        <x:v>EEHZL1V470R</x:v>
-      </x:c>
-      <x:c r="F15" s="9" t="str"/>
+        <x:v>EEHZA1V470P</x:v>
+      </x:c>
+      <x:c r="F15" s="9" t="str">
+        <x:v>C178639</x:v>
+      </x:c>
       <x:c r="G15" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H15" s="14" t="str">
-        <x:v>NO CONFIRMED SKU</x:v>
+        <x:v>CANDIDATE / 105C REVIEW</x:v>
       </x:c>
       <x:c r="I15" s="9" t="str">
-        <x:v>Check ESR, voltage and physical fit</x:v>
+        <x:v>35V/47u/60mΩ; old 135C to 105C downgrade; verify land pattern, polarity and heat</x:v>
       </x:c>
       <x:c r="J15" s="9" t="str">
         <x:v>YES</x:v>
@@ -906,16 +925,20 @@
       <x:c r="D17" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E17" s="9" t="str"/>
-      <x:c r="F17" s="9" t="str"/>
+      <x:c r="E17" s="9" t="str">
+        <x:v>1210X476M250CT</x:v>
+      </x:c>
+      <x:c r="F17" s="9" t="str">
+        <x:v>C3848311</x:v>
+      </x:c>
       <x:c r="G17" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H17" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / DC BIAS REVIEW</x:v>
       </x:c>
       <x:c r="I17" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Walsin X5R 47uF 25V 1210; verify effective µF at 12.5V &amp; stock</x:v>
       </x:c>
       <x:c r="J17" s="9" t="str">
         <x:v>YES</x:v>
@@ -934,16 +957,20 @@
       <x:c r="D18" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E18" s="9" t="str"/>
-      <x:c r="F18" s="9" t="str"/>
+      <x:c r="E18" s="9" t="str">
+        <x:v>1210X476M250CT</x:v>
+      </x:c>
+      <x:c r="F18" s="9" t="str">
+        <x:v>C3848311</x:v>
+      </x:c>
       <x:c r="G18" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H18" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / DC BIAS REVIEW</x:v>
       </x:c>
       <x:c r="I18" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Walsin X5R 47uF 25V 1210; verify effective µF at 12.5V &amp; stock</x:v>
       </x:c>
       <x:c r="J18" s="9" t="str">
         <x:v>YES</x:v>
@@ -962,16 +989,20 @@
       <x:c r="D19" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E19" s="9" t="str"/>
-      <x:c r="F19" s="9" t="str"/>
+      <x:c r="E19" s="9" t="str">
+        <x:v>1210X476M250CT</x:v>
+      </x:c>
+      <x:c r="F19" s="9" t="str">
+        <x:v>C3848311</x:v>
+      </x:c>
       <x:c r="G19" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H19" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / DC BIAS REVIEW</x:v>
       </x:c>
       <x:c r="I19" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Walsin X5R 47uF 25V 1210; verify effective µF at 12.5V &amp; stock</x:v>
       </x:c>
       <x:c r="J19" s="9" t="str">
         <x:v>YES</x:v>
@@ -991,17 +1022,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
-        <x:v>250AVHT221M0608</x:v>
-      </x:c>
-      <x:c r="F20" s="9" t="str"/>
+        <x:v>MA25V220M6X8</x:v>
+      </x:c>
+      <x:c r="F20" s="9" t="str">
+        <x:v>C46550464</x:v>
+      </x:c>
       <x:c r="G20" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
-        <x:v>NO CONFIRMED SKU</x:v>
+        <x:v>CANDIDATE / LOOP REVIEW</x:v>
       </x:c>
       <x:c r="I20" s="9" t="str">
-        <x:v>Verify ESR, ripple current and loop stability</x:v>
+        <x:v>25V/220u, 28 vs 24mΩ; 105C vs original 125C; stability and land pattern</x:v>
       </x:c>
       <x:c r="J20" s="9" t="str">
         <x:v>YES</x:v>
@@ -1048,16 +1081,20 @@
       <x:c r="D22" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E22" s="9" t="str"/>
-      <x:c r="F22" s="9" t="str"/>
+      <x:c r="E22" s="9" t="str">
+        <x:v>1210X476M250CT</x:v>
+      </x:c>
+      <x:c r="F22" s="9" t="str">
+        <x:v>C3848311</x:v>
+      </x:c>
       <x:c r="G22" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H22" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / DC BIAS REVIEW</x:v>
       </x:c>
       <x:c r="I22" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>Walsin X5R 47uF 25V 1210; verify effective µF at 12.5V &amp; stock</x:v>
       </x:c>
       <x:c r="J22" s="9" t="str">
         <x:v>YES</x:v>
@@ -1217,17 +1254,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
-        <x:v>1206SFS300F/32</x:v>
-      </x:c>
-      <x:c r="F28" s="9" t="str"/>
+        <x:v>0468003.NRHF</x:v>
+      </x:c>
+      <x:c r="F28" s="9" t="str">
+        <x:v>C41342</x:v>
+      </x:c>
       <x:c r="G28" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H28" s="14" t="str">
-        <x:v>NO CONFIRMED SKU</x:v>
+        <x:v>CANDIDATE / FUSE DERATING</x:v>
       </x:c>
       <x:c r="I28" s="9" t="str">
-        <x:v>Match voltage/current, I-squared-t and derating</x:v>
+        <x:v>3A/32V, I²t 1.27 vs 1.20 A²s; 90C vs original 125C; fuse curve review</x:v>
       </x:c>
       <x:c r="J28" s="9" t="str">
         <x:v>YES</x:v>
@@ -1598,16 +1637,20 @@
       <x:c r="D41" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E41" s="9" t="str"/>
-      <x:c r="F41" s="9" t="str"/>
+      <x:c r="E41" s="9" t="str">
+        <x:v>RT0603BRD07100KL</x:v>
+      </x:c>
+      <x:c r="F41" s="9" t="str">
+        <x:v>C122538</x:v>
+      </x:c>
       <x:c r="G41" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H41" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / 0.1% VERIFY</x:v>
       </x:c>
       <x:c r="I41" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>100k 0.1% 25ppm thin film; check stock and resistor power</x:v>
       </x:c>
       <x:c r="J41" s="9" t="str">
         <x:v>YES</x:v>
@@ -1626,16 +1669,20 @@
       <x:c r="D42" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E42" s="9" t="str"/>
-      <x:c r="F42" s="9" t="str"/>
+      <x:c r="E42" s="9" t="str">
+        <x:v>RT0603BRD078K66L</x:v>
+      </x:c>
+      <x:c r="F42" s="9" t="str">
+        <x:v>C861591</x:v>
+      </x:c>
       <x:c r="G42" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H42" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / 0.1% VERIFY</x:v>
       </x:c>
       <x:c r="I42" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>8.66k 0.1% 25ppm thin film; check stock and resistor power</x:v>
       </x:c>
       <x:c r="J42" s="9" t="str">
         <x:v>YES</x:v>
@@ -2503,13 +2550,13 @@
         <x:v>C18</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>EEHZL1V470R_47u</x:v>
+        <x:v>EEHZA1V470P_47u</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>CP_Elec_5x5.8</x:v>
+        <x:v>CP_Elec_6.3x5.8</x:v>
       </x:c>
       <x:c r="D14" s="17" t="n">
-        <x:v>62</x:v>
+        <x:v>61.5</x:v>
       </x:c>
       <x:c r="E14" s="17" t="n">
         <x:v>-48</x:v>
@@ -2524,7 +2571,7 @@
         <x:v>top</x:v>
       </x:c>
       <x:c r="I14" s="12" t="str">
-        <x:v>CHECK orientation / center</x:v>
+        <x:v>CHECK POLARITY / 6.3mm PACKAGE / CENTER</x:v>
       </x:c>
     </x:row>
     <x:row r="15">

</xml_diff>

<commit_message>
Rev B: map 53 SMT candidate C-codes and audit power copper necks (NO-GO)
</commit_message>
<xml_diff>
--- a/manufacturing/Rev_B/REVIEW_ONLY_NOT_FOR_FAB/FT2D_RevB_SMT_sourcing_DRAFT.xlsx
+++ b/manufacturing/Rev_B/REVIEW_ONLY_NOT_FOR_FAB/FT2D_RevB_SMT_sourcing_DRAFT.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="R4212f2852f1f4ec3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM review" sheetId="2" r:id="R038f215f37004454"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPL preview" sheetId="3" r:id="R3c5e969274e64cce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="R52bad606bf1c4cc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM review" sheetId="2" r:id="R95cce85eb4c24a8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPL preview" sheetId="3" r:id="R8cc6e737ecd5463f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -394,7 +394,7 @@
         <x:v>JLCPCB sourcing</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
-        <x:v>Candidate C-codes for critical/R-C parts; most passives not sourced; stock unverified</x:v>
+        <x:v>53/53 SMT refs mapped to 36 candidate C-codes; 0 approved; stock and physical compatibility NOT verified</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -410,12 +410,12 @@
         <x:v>Placement file</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
-        <x:v>53 SMT positions; -90deg USB-C placement &amp; Y sign need JLC review</x:v>
+        <x:v>53 native KiCad positions + candidate JLC CSV previews; Y sign &amp; rotation need JLC visual approval</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="8" t="str">
-        <x:v>For planning/preview only: this is NOT a release BOM/CPL.</x:v>
+        <x:v>53/53 candidate SKU coverage DOES NOT MEAN fabrication approval; 3A and JLC SMT/thermal gates remain open.</x:v>
       </x:c>
       <x:c r="B14"/>
     </x:row>
@@ -485,16 +485,20 @@
       <x:c r="D2" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E2" s="9" t="str"/>
-      <x:c r="F2" s="9" t="str"/>
+      <x:c r="E2" s="9" t="str">
+        <x:v>C1608X7R1A105K080AC</x:v>
+      </x:c>
+      <x:c r="F2" s="9" t="str">
+        <x:v>C5332007</x:v>
+      </x:c>
       <x:c r="G2" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H2" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / BIAS / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I2" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对 DC 偏压有效容值、X7R/温度和封装；JLC 动态库存待确认</x:v>
       </x:c>
       <x:c r="J2" s="9" t="str">
         <x:v>YES</x:v>
@@ -513,16 +517,20 @@
       <x:c r="D3" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E3" s="9" t="str"/>
-      <x:c r="F3" s="9" t="str"/>
+      <x:c r="E3" s="9" t="str">
+        <x:v>C1608X7R1A105K080AC</x:v>
+      </x:c>
+      <x:c r="F3" s="9" t="str">
+        <x:v>C5332007</x:v>
+      </x:c>
       <x:c r="G3" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H3" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / BIAS / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I3" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对 DC 偏压有效容值、X7R/温度和封装；JLC 动态库存待确认</x:v>
       </x:c>
       <x:c r="J3" s="9" t="str">
         <x:v>YES</x:v>
@@ -541,16 +549,20 @@
       <x:c r="D4" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E4" s="9" t="str"/>
-      <x:c r="F4" s="9" t="str"/>
+      <x:c r="E4" s="9" t="str">
+        <x:v>CL21B105KAFNFNE</x:v>
+      </x:c>
+      <x:c r="F4" s="9" t="str">
+        <x:v>C1712</x:v>
+      </x:c>
       <x:c r="G4" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H4" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / BIAS / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I4" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对 DC 偏压有效容值、X7R/温度和封装；JLC 动态库存待确认</x:v>
       </x:c>
       <x:c r="J4" s="9" t="str">
         <x:v>YES</x:v>
@@ -569,16 +581,20 @@
       <x:c r="D5" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E5" s="9" t="str"/>
-      <x:c r="F5" s="9" t="str"/>
+      <x:c r="E5" s="9" t="str">
+        <x:v>C1608X7R1H473KT000N</x:v>
+      </x:c>
+      <x:c r="F5" s="9" t="str">
+        <x:v>C380378</x:v>
+      </x:c>
       <x:c r="G5" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H5" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J5" s="9" t="str">
         <x:v>YES</x:v>
@@ -597,16 +613,20 @@
       <x:c r="D6" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E6" s="9" t="str"/>
-      <x:c r="F6" s="9" t="str"/>
+      <x:c r="E6" s="9" t="str">
+        <x:v>CL21B105KAFNFNE</x:v>
+      </x:c>
+      <x:c r="F6" s="9" t="str">
+        <x:v>C1712</x:v>
+      </x:c>
       <x:c r="G6" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H6" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / BIAS / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I6" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对 DC 偏压有效容值、X7R/温度和封装；JLC 动态库存待确认</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
         <x:v>YES</x:v>
@@ -625,16 +645,20 @@
       <x:c r="D7" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E7" s="9" t="str"/>
-      <x:c r="F7" s="9" t="str"/>
+      <x:c r="E7" s="9" t="str">
+        <x:v>CGA3E1X7R1C105K080AC</x:v>
+      </x:c>
+      <x:c r="F7" s="9" t="str">
+        <x:v>C194115</x:v>
+      </x:c>
       <x:c r="G7" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H7" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / BIAS / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I7" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对 DC 偏压有效容值、X7R/温度和封装；JLC 动态库存待确认</x:v>
       </x:c>
       <x:c r="J7" s="9" t="str">
         <x:v>YES</x:v>
@@ -681,16 +705,20 @@
       <x:c r="D9" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E9" s="9" t="str"/>
-      <x:c r="F9" s="9" t="str"/>
+      <x:c r="E9" s="9" t="str">
+        <x:v>C1608X7R1H104K080AE</x:v>
+      </x:c>
+      <x:c r="F9" s="9" t="str">
+        <x:v>C2167477</x:v>
+      </x:c>
       <x:c r="G9" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H9" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I9" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J9" s="9" t="str">
         <x:v>YES</x:v>
@@ -709,16 +737,20 @@
       <x:c r="D10" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E10" s="9" t="str"/>
-      <x:c r="F10" s="9" t="str"/>
+      <x:c r="E10" s="9" t="str">
+        <x:v>C1608X7R1H104K080AE</x:v>
+      </x:c>
+      <x:c r="F10" s="9" t="str">
+        <x:v>C2167477</x:v>
+      </x:c>
       <x:c r="G10" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H10" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I10" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
         <x:v>YES</x:v>
@@ -897,16 +929,20 @@
       <x:c r="D16" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E16" s="9" t="str"/>
-      <x:c r="F16" s="9" t="str"/>
+      <x:c r="E16" s="9" t="str">
+        <x:v>GCM188R71E104KA57D</x:v>
+      </x:c>
+      <x:c r="F16" s="9" t="str">
+        <x:v>C85861</x:v>
+      </x:c>
       <x:c r="G16" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H16" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I16" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J16" s="9" t="str">
         <x:v>YES</x:v>
@@ -1053,16 +1089,20 @@
       <x:c r="D21" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E21" s="9" t="str"/>
-      <x:c r="F21" s="9" t="str"/>
+      <x:c r="E21" s="9" t="str">
+        <x:v>GCM188R71E104KA57D</x:v>
+      </x:c>
+      <x:c r="F21" s="9" t="str">
+        <x:v>C85861</x:v>
+      </x:c>
       <x:c r="G21" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H21" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I21" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J21" s="9" t="str">
         <x:v>YES</x:v>
@@ -1113,16 +1153,20 @@
       <x:c r="D23" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E23" s="9" t="str"/>
-      <x:c r="F23" s="9" t="str"/>
+      <x:c r="E23" s="9" t="str">
+        <x:v>GCM188R71E104KA57D</x:v>
+      </x:c>
+      <x:c r="F23" s="9" t="str">
+        <x:v>C85861</x:v>
+      </x:c>
       <x:c r="G23" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H23" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I23" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J23" s="9" t="str">
         <x:v>YES</x:v>
@@ -1141,16 +1185,20 @@
       <x:c r="D24" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E24" s="9" t="str"/>
-      <x:c r="F24" s="9" t="str"/>
+      <x:c r="E24" s="9" t="str">
+        <x:v>GRM1885C1H332JA01D</x:v>
+      </x:c>
+      <x:c r="F24" s="9" t="str">
+        <x:v>C77036</x:v>
+      </x:c>
       <x:c r="G24" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H24" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I24" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J24" s="9" t="str">
         <x:v>YES</x:v>
@@ -1169,16 +1217,20 @@
       <x:c r="D25" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E25" s="9" t="str"/>
-      <x:c r="F25" s="9" t="str"/>
+      <x:c r="E25" s="9" t="str">
+        <x:v>GRM1885C1H222JA01D</x:v>
+      </x:c>
+      <x:c r="F25" s="9" t="str">
+        <x:v>C77033</x:v>
+      </x:c>
       <x:c r="G25" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H25" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I25" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J25" s="9" t="str">
         <x:v>YES</x:v>
@@ -1197,16 +1249,20 @@
       <x:c r="D26" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E26" s="9" t="str"/>
-      <x:c r="F26" s="9" t="str"/>
+      <x:c r="E26" s="9" t="str">
+        <x:v>ESDA25P35-1U1M</x:v>
+      </x:c>
+      <x:c r="F26" s="9" t="str">
+        <x:v>C1974707</x:v>
+      </x:c>
       <x:c r="G26" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H26" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / TVS_PINOUT / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I26" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对 TVS 极性/引脚分配、封装方向及 ESD 工作电压</x:v>
       </x:c>
       <x:c r="J26" s="9" t="str">
         <x:v>YES</x:v>
@@ -1225,16 +1281,20 @@
       <x:c r="D27" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E27" s="9" t="str"/>
-      <x:c r="F27" s="9" t="str"/>
+      <x:c r="E27" s="9" t="str">
+        <x:v>ESDA25W</x:v>
+      </x:c>
+      <x:c r="F27" s="9" t="str">
+        <x:v>C2935152</x:v>
+      </x:c>
       <x:c r="G27" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H27" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / TVS_PINOUT / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I27" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对 TVS 极性/引脚分配、封装方向及 ESD 工作电压</x:v>
       </x:c>
       <x:c r="J27" s="9" t="str">
         <x:v>YES</x:v>
@@ -1441,16 +1501,20 @@
       <x:c r="D34" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E34" s="9" t="str"/>
-      <x:c r="F34" s="9" t="str"/>
+      <x:c r="E34" s="9" t="str">
+        <x:v>RC0603FR-0710KL</x:v>
+      </x:c>
+      <x:c r="F34" s="9" t="str">
+        <x:v>C98220</x:v>
+      </x:c>
       <x:c r="G34" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H34" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I34" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J34" s="9" t="str">
         <x:v>YES</x:v>
@@ -1469,16 +1533,20 @@
       <x:c r="D35" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E35" s="9" t="str"/>
-      <x:c r="F35" s="9" t="str"/>
+      <x:c r="E35" s="9" t="str">
+        <x:v>RC0603FR-074K7L</x:v>
+      </x:c>
+      <x:c r="F35" s="9" t="str">
+        <x:v>C99782</x:v>
+      </x:c>
       <x:c r="G35" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H35" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I35" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J35" s="9" t="str">
         <x:v>YES</x:v>
@@ -1497,16 +1565,20 @@
       <x:c r="D36" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E36" s="9" t="str"/>
-      <x:c r="F36" s="9" t="str"/>
+      <x:c r="E36" s="9" t="str">
+        <x:v>RC0603FR-074K7L</x:v>
+      </x:c>
+      <x:c r="F36" s="9" t="str">
+        <x:v>C99782</x:v>
+      </x:c>
       <x:c r="G36" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H36" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I36" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J36" s="9" t="str">
         <x:v>YES</x:v>
@@ -1525,16 +1597,20 @@
       <x:c r="D37" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E37" s="9" t="str"/>
-      <x:c r="F37" s="9" t="str"/>
+      <x:c r="E37" s="9" t="str">
+        <x:v>RC0603FR-071KL</x:v>
+      </x:c>
+      <x:c r="F37" s="9" t="str">
+        <x:v>C22548</x:v>
+      </x:c>
       <x:c r="G37" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H37" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I37" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J37" s="9" t="str">
         <x:v>YES</x:v>
@@ -1553,16 +1629,20 @@
       <x:c r="D38" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E38" s="9" t="str"/>
-      <x:c r="F38" s="9" t="str"/>
+      <x:c r="E38" s="9" t="str">
+        <x:v>RC0603FR-1322KP</x:v>
+      </x:c>
+      <x:c r="F38" s="9" t="str">
+        <x:v>C5717132</x:v>
+      </x:c>
       <x:c r="G38" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H38" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I38" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J38" s="9" t="str">
         <x:v>YES</x:v>
@@ -1581,16 +1661,20 @@
       <x:c r="D39" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E39" s="9" t="str"/>
-      <x:c r="F39" s="9" t="str"/>
+      <x:c r="E39" s="9" t="str">
+        <x:v>RC0603FR-07470RL</x:v>
+      </x:c>
+      <x:c r="F39" s="9" t="str">
+        <x:v>C114669</x:v>
+      </x:c>
       <x:c r="G39" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H39" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I39" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J39" s="9" t="str">
         <x:v>YES</x:v>
@@ -1609,16 +1693,20 @@
       <x:c r="D40" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E40" s="9" t="str"/>
-      <x:c r="F40" s="9" t="str"/>
+      <x:c r="E40" s="9" t="str">
+        <x:v>RC0603FR-07100KL</x:v>
+      </x:c>
+      <x:c r="F40" s="9" t="str">
+        <x:v>C14675</x:v>
+      </x:c>
       <x:c r="G40" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H40" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I40" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J40" s="9" t="str">
         <x:v>YES</x:v>
@@ -1729,16 +1817,20 @@
       <x:c r="D44" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E44" s="9" t="str"/>
-      <x:c r="F44" s="9" t="str"/>
+      <x:c r="E44" s="9" t="str">
+        <x:v>RC0603FR-07100KL</x:v>
+      </x:c>
+      <x:c r="F44" s="9" t="str">
+        <x:v>C14675</x:v>
+      </x:c>
       <x:c r="G44" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H44" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I44" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J44" s="9" t="str">
         <x:v>YES</x:v>
@@ -1757,16 +1849,20 @@
       <x:c r="D45" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E45" s="9" t="str"/>
-      <x:c r="F45" s="9" t="str"/>
+      <x:c r="E45" s="9" t="str">
+        <x:v>AC0603FR-0733K2L</x:v>
+      </x:c>
+      <x:c r="F45" s="9" t="str">
+        <x:v>C227824</x:v>
+      </x:c>
       <x:c r="G45" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H45" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I45" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J45" s="9" t="str">
         <x:v>YES</x:v>
@@ -1785,16 +1881,20 @@
       <x:c r="D46" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E46" s="9" t="str"/>
-      <x:c r="F46" s="9" t="str"/>
+      <x:c r="E46" s="9" t="str">
+        <x:v>RMCF0603FT133K</x:v>
+      </x:c>
+      <x:c r="F46" s="9" t="str">
+        <x:v>C2484234</x:v>
+      </x:c>
       <x:c r="G46" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H46" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I46" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J46" s="9" t="str">
         <x:v>YES</x:v>
@@ -1813,16 +1913,20 @@
       <x:c r="D47" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E47" s="9" t="str"/>
-      <x:c r="F47" s="9" t="str"/>
+      <x:c r="E47" s="9" t="str">
+        <x:v>RC0603FR-0710KL</x:v>
+      </x:c>
+      <x:c r="F47" s="9" t="str">
+        <x:v>C98220</x:v>
+      </x:c>
       <x:c r="G47" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H47" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I47" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J47" s="9" t="str">
         <x:v>YES</x:v>
@@ -1841,16 +1945,20 @@
       <x:c r="D48" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E48" s="9" t="str"/>
-      <x:c r="F48" s="9" t="str"/>
+      <x:c r="E48" s="9" t="str">
+        <x:v>RC0603JR-070RL</x:v>
+      </x:c>
+      <x:c r="F48" s="9" t="str">
+        <x:v>C95177</x:v>
+      </x:c>
       <x:c r="G48" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H48" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / ZERO_OHM / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I48" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对零欧电阻额定工作电流、封装和库存</x:v>
       </x:c>
       <x:c r="J48" s="9" t="str">
         <x:v>YES</x:v>
@@ -1869,16 +1977,20 @@
       <x:c r="D49" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E49" s="9" t="str"/>
-      <x:c r="F49" s="9" t="str"/>
+      <x:c r="E49" s="9" t="str">
+        <x:v>RTT034703FTP</x:v>
+      </x:c>
+      <x:c r="F49" s="9" t="str">
+        <x:v>C103658</x:v>
+      </x:c>
       <x:c r="G49" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H49" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I49" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J49" s="9" t="str">
         <x:v>YES</x:v>
@@ -1897,16 +2009,20 @@
       <x:c r="D50" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E50" s="9" t="str"/>
-      <x:c r="F50" s="9" t="str"/>
+      <x:c r="E50" s="9" t="str">
+        <x:v>RC0603FR-07100KL</x:v>
+      </x:c>
+      <x:c r="F50" s="9" t="str">
+        <x:v>C14675</x:v>
+      </x:c>
       <x:c r="G50" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H50" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I50" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J50" s="9" t="str">
         <x:v>YES</x:v>
@@ -1925,16 +2041,20 @@
       <x:c r="D51" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E51" s="9" t="str"/>
-      <x:c r="F51" s="9" t="str"/>
+      <x:c r="E51" s="9" t="str">
+        <x:v>RN73H1JTTD1013F100</x:v>
+      </x:c>
+      <x:c r="F51" s="9" t="str">
+        <x:v>C4016651</x:v>
+      </x:c>
       <x:c r="G51" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H51" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / EXACT_101K_STOCK / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I51" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>101kΩ 原设计值无需替换；C4016651 在 LCSC 可查，须核对 JLC 是否支持 SMT 和库存</x:v>
       </x:c>
       <x:c r="J51" s="9" t="str">
         <x:v>YES</x:v>
@@ -1953,16 +2073,20 @@
       <x:c r="D52" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E52" s="9" t="str"/>
-      <x:c r="F52" s="9" t="str"/>
+      <x:c r="E52" s="9" t="str">
+        <x:v>RC0603FR-0710KL</x:v>
+      </x:c>
+      <x:c r="F52" s="9" t="str">
+        <x:v>C98220</x:v>
+      </x:c>
       <x:c r="G52" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H52" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I52" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J52" s="9" t="str">
         <x:v>YES</x:v>
@@ -1981,16 +2105,20 @@
       <x:c r="D53" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E53" s="9" t="str"/>
-      <x:c r="F53" s="9" t="str"/>
+      <x:c r="E53" s="9" t="str">
+        <x:v>RC0603FR-07100KL</x:v>
+      </x:c>
+      <x:c r="F53" s="9" t="str">
+        <x:v>C14675</x:v>
+      </x:c>
       <x:c r="G53" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H53" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I53" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J53" s="9" t="str">
         <x:v>YES</x:v>
@@ -2009,16 +2137,20 @@
       <x:c r="D54" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E54" s="9" t="str"/>
-      <x:c r="F54" s="9" t="str"/>
+      <x:c r="E54" s="9" t="str">
+        <x:v>RC0603FR-0712KL</x:v>
+      </x:c>
+      <x:c r="F54" s="9" t="str">
+        <x:v>C114659</x:v>
+      </x:c>
       <x:c r="G54" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H54" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I54" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J54" s="9" t="str">
         <x:v>YES</x:v>
@@ -2037,16 +2169,20 @@
       <x:c r="D55" s="10" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E55" s="9" t="str"/>
-      <x:c r="F55" s="9" t="str"/>
+      <x:c r="E55" s="9" t="str">
+        <x:v>0603WAF8200T5E</x:v>
+      </x:c>
+      <x:c r="F55" s="9" t="str">
+        <x:v>C23253</x:v>
+      </x:c>
       <x:c r="G55" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H55" s="12" t="str">
-        <x:v>SKU NOT ASSIGNED</x:v>
+        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I55" s="9" t="str">
-        <x:v>Verify rating, tolerance, land pattern and stock</x:v>
+        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
       </x:c>
       <x:c r="J55" s="9" t="str">
         <x:v>YES</x:v>

</xml_diff>

<commit_message>
Rev B: stitch U3 power copper and upgrade output bypass; refresh JLC review QA (NO-GO)
</commit_message>
<xml_diff>
--- a/manufacturing/Rev_B/REVIEW_ONLY_NOT_FOR_FAB/FT2D_RevB_SMT_sourcing_DRAFT.xlsx
+++ b/manufacturing/Rev_B/REVIEW_ONLY_NOT_FOR_FAB/FT2D_RevB_SMT_sourcing_DRAFT.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="R52bad606bf1c4cc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM review" sheetId="2" r:id="R95cce85eb4c24a8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPL preview" sheetId="3" r:id="R8cc6e737ecd5463f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="Rda36183e9dfc445e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM review" sheetId="2" r:id="R363a0dac48e94c84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPL preview" sheetId="3" r:id="Rb5dbc608d8404620"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -394,7 +394,7 @@
         <x:v>JLCPCB sourcing</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
-        <x:v>53/53 SMT refs mapped to 36 candidate C-codes; 0 approved; stock and physical compatibility NOT verified</x:v>
+        <x:v>53/53 SMT refs; 37 candidate MPNs; 0 approved; C26 now 2.2uF/25V</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1154,19 +1154,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
-        <x:v>GCM188R71E104KA57D</x:v>
+        <x:v>GRM188Z71E225KE43D</x:v>
       </x:c>
       <x:c r="F23" s="9" t="str">
-        <x:v>C85861</x:v>
+        <x:v>C415535</x:v>
       </x:c>
       <x:c r="G23" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H23" s="12" t="str">
-        <x:v>CANDIDATE / NORMAL / NOT APPROVED</x:v>
+        <x:v>CANDIDATE / OUT_DECOUPLING_BIAS / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I23" s="9" t="str">
-        <x:v>核对厂家规格、电压/功率/尺寸与嘉立创当前 SMT 料号、库存及最小采购量</x:v>
+        <x:v>U3 输出去耦从 100nF 改 2.2uF/25V X7R；须核对 12.5V DC-bias 有效容值、靠近 OUT 引脚与库存</x:v>
       </x:c>
       <x:c r="J23" s="9" t="str">
         <x:v>YES</x:v>

</xml_diff>

<commit_message>
Rev B: qualify JLC SMT 102k OVLO resistor and refresh fab preview artifacts (NO-GO)
</commit_message>
<xml_diff>
--- a/manufacturing/Rev_B/REVIEW_ONLY_NOT_FOR_FAB/FT2D_RevB_SMT_sourcing_DRAFT.xlsx
+++ b/manufacturing/Rev_B/REVIEW_ONLY_NOT_FOR_FAB/FT2D_RevB_SMT_sourcing_DRAFT.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="Rda36183e9dfc445e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM review" sheetId="2" r:id="R363a0dac48e94c84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPL preview" sheetId="3" r:id="Rb5dbc608d8404620"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ReadMe" sheetId="1" r:id="R07db72af1c7b4929"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM review" sheetId="2" r:id="Rc399c48114f64f02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CPL preview" sheetId="3" r:id="R6a037602850a4654"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -394,7 +394,7 @@
         <x:v>JLCPCB sourcing</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
-        <x:v>53/53 SMT refs; 37 candidate MPNs; 0 approved; C26 now 2.2uF/25V</x:v>
+        <x:v>53/53 SMT refs; 37 candidate MPNs; 0 approved; C26 2.2uF/25V; R22 102k/C861068</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2042,19 +2042,19 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="E51" s="9" t="str">
-        <x:v>RN73H1JTTD1013F100</x:v>
+        <x:v>RT0603BRD07102KL</x:v>
       </x:c>
       <x:c r="F51" s="9" t="str">
-        <x:v>C4016651</x:v>
+        <x:v>C861068</x:v>
       </x:c>
       <x:c r="G51" s="9" t="str">
         <x:v>SMT</x:v>
       </x:c>
       <x:c r="H51" s="12" t="str">
-        <x:v>CANDIDATE / EXACT_101K_STOCK / NOT APPROVED</x:v>
+        <x:v>CANDIDATE / OVLO_102K_SMT_CONFIRMED / NOT APPROVED</x:v>
       </x:c>
       <x:c r="I51" s="9" t="str">
-        <x:v>101kΩ 原设计值无需替换；C4016651 在 LCSC 可查，须核对 JLC 是否支持 SMT 和库存</x:v>
+        <x:v>R22 改 102kΩ ±0.1% Yageo C861068；典型 OVLO 由 13.32V 调为 13.44V；JLC 列 SMT，实时库存、过压实测待审</x:v>
       </x:c>
       <x:c r="J51" s="9" t="str">
         <x:v>YES</x:v>

</xml_diff>